<commit_message>
📅 日报更新 2026-09-05 03:05
</commit_message>
<xml_diff>
--- a/data/exports/黄老师/dist_order_2026-09-05.xlsx
+++ b/data/exports/黄老师/dist_order_2026-09-05.xlsx
@@ -125,11 +125,11 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="0">
-        <v>50058017</v>
+        <v>50074867</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>索描贾师＃壹皇贰金山玉旗🇨🇳</t>
+          <t>美好人生</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:16:49</t>
+          <t>2026-09-05 10:19:59</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -164,7 +164,7 @@
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J2" s="0" t="inlineStr">
@@ -185,11 +185,11 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="0">
-        <v>50057895</v>
+        <v>50074273</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>南雪</t>
+          <t>周利平</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -214,7 +214,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:12:32</t>
+          <t>2026-09-05 10:02:26</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -240,21 +240,16 @@
       <c r="L3" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N3" s="0" t="inlineStr">
-        <is>
-          <t>镇江</t>
         </is>
       </c>
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="0">
-        <v>50057857</v>
+        <v>50074103</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>可心</t>
+          <t>赵香荣</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -279,7 +274,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:55</t>
+          <t>2026-09-05 09:58:29</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -310,11 +305,11 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="0">
-        <v>50057854</v>
+        <v>50074078</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>张苏龙</t>
+          <t>长风渡℡明</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -339,7 +334,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:51</t>
+          <t>2026-09-05 09:57:49</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -370,11 +365,11 @@
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="0">
-        <v>50057852</v>
+        <v>50074077</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>？</t>
+          <t>海阔天空bi</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -399,7 +394,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:43</t>
+          <t>2026-09-05 09:57:47</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -430,11 +425,11 @@
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="0">
-        <v>50057841</v>
+        <v>50074076</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>向往的生活-电信号</t>
+          <t>枫叶红</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -459,7 +454,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:09</t>
+          <t>2026-09-05 09:57:47</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -490,11 +485,11 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="0">
-        <v>50057839</v>
+        <v>50074071</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>金盏花</t>
+          <t>思缘</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -519,7 +514,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:03</t>
+          <t>2026-09-05 09:57:35</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -550,11 +545,11 @@
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="0">
-        <v>50032697</v>
+        <v>50074067</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>小米. ᩚ</t>
+          <t>悠然</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -579,7 +574,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:24:13</t>
+          <t>2026-09-05 09:57:25</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -589,7 +584,7 @@
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
@@ -610,11 +605,11 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="0">
-        <v>50032693</v>
+        <v>50058017</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>海岸</t>
+          <t>索描贾师＃壹皇贰金山玉旗🇨🇳</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -639,7 +634,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:24:11</t>
+          <t>2026-09-04 23:16:49</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
@@ -649,7 +644,7 @@
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J10" s="0" t="inlineStr">
@@ -670,11 +665,11 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="0">
-        <v>50032683</v>
+        <v>50057895</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>陆建军</t>
+          <t>南雪</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -699,7 +694,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:23:53</t>
+          <t>2026-09-04 23:12:32</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -709,7 +704,7 @@
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J11" s="0" t="inlineStr">
@@ -725,16 +720,21 @@
       <c r="L11" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N11" s="0" t="inlineStr">
+        <is>
+          <t>镇江</t>
         </is>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="0">
-        <v>50015883</v>
+        <v>50057857</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>A00金华义乌叉车出租电15268650979</t>
+          <t>可心</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:18:02</t>
+          <t>2026-09-04 23:10:55</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
@@ -790,11 +790,11 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="0">
-        <v>50015882</v>
+        <v>50057854</v>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>建程仓储中心 张川</t>
+          <t>张苏龙</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:18:02</t>
+          <t>2026-09-04 23:10:51</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
@@ -850,11 +850,11 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="0">
-        <v>50015784</v>
+        <v>50057852</v>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>天空</t>
+          <t>？</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:41</t>
+          <t>2026-09-04 23:10:43</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -910,11 +910,11 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="0">
-        <v>50015778</v>
+        <v>50057841</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>小龙女</t>
+          <t>向往的生活-电信号</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -939,7 +939,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:21</t>
+          <t>2026-09-04 23:10:09</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -970,11 +970,11 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="0">
-        <v>50015776</v>
+        <v>50057839</v>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>桥梁</t>
+          <t>金盏花</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:15</t>
+          <t>2026-09-04 23:10:03</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
@@ -1030,11 +1030,11 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="0">
-        <v>50015775</v>
+        <v>50032697</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>彩云之南</t>
+          <t>小米. ᩚ</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:13</t>
+          <t>2026-09-04 12:24:13</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J17" s="0" t="inlineStr">
@@ -1090,11 +1090,11 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="0">
-        <v>50015774</v>
+        <v>50032693</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>楊精蓄銳༒</t>
+          <t>海岸</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:11</t>
+          <t>2026-09-04 12:24:11</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
@@ -1150,11 +1150,11 @@
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="0">
-        <v>50015772</v>
+        <v>50032683</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>不倒翁</t>
+          <t>陆建军</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:07</t>
+          <t>2026-09-04 12:23:53</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="I19" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J19" s="0" t="inlineStr">
@@ -1210,11 +1210,11 @@
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="0">
-        <v>50015770</v>
+        <v>50015883</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>一江春水</t>
+          <t>A00金华义乌叉车出租电15268650979</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:05</t>
+          <t>2026-09-03 23:18:02</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J20" s="0" t="inlineStr">
@@ -1270,11 +1270,11 @@
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="0">
-        <v>50015767</v>
+        <v>50015882</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>微笑</t>
+          <t>建程仓储中心 张川</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:03</t>
+          <t>2026-09-03 23:18:02</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
@@ -1330,11 +1330,11 @@
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="0">
-        <v>50015763</v>
+        <v>50015784</v>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>北斗星</t>
+          <t>天空</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:09:39</t>
+          <t>2026-09-03 23:10:41</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
@@ -1390,11 +1390,11 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="0">
-        <v>49989442</v>
+        <v>50015778</v>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>冬梅花儿开王丽君</t>
+          <t>小龙女</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:43</t>
+          <t>2026-09-03 23:10:21</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="I23" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J23" s="0" t="inlineStr">
@@ -1450,11 +1450,11 @@
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="0">
-        <v>49989431</v>
+        <v>50015776</v>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>风声</t>
+          <t>桥梁</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:25</t>
+          <t>2026-09-03 23:10:15</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="I24" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J24" s="0" t="inlineStr">
@@ -1510,11 +1510,11 @@
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="0">
-        <v>49989419</v>
+        <v>50015775</v>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>胡宾</t>
+          <t>彩云之南</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:13</t>
+          <t>2026-09-03 23:10:13</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="I25" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J25" s="0" t="inlineStr">
@@ -1570,11 +1570,11 @@
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="0">
-        <v>49989410</v>
+        <v>50015774</v>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>永远</t>
+          <t>楊精蓄銳༒</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:03</t>
+          <t>2026-09-03 23:10:11</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="I26" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J26" s="0" t="inlineStr">
@@ -1630,11 +1630,11 @@
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="0">
-        <v>49984259</v>
+        <v>50015772</v>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>好运包张</t>
+          <t>不倒翁</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:55:37</t>
+          <t>2026-09-03 23:10:07</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="I27" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J27" s="0" t="inlineStr">
@@ -1690,11 +1690,11 @@
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="0">
-        <v>49984055</v>
+        <v>50015770</v>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>点点星辰</t>
+          <t>一江春水</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:49:33</t>
+          <t>2026-09-03 23:10:05</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
@@ -1750,11 +1750,11 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" s="0">
-        <v>49983134</v>
+        <v>50015767</v>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>Zhangrruzhen张如真</t>
+          <t>微笑</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:25:21</t>
+          <t>2026-09-03 23:10:03</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="I29" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J29" s="0" t="inlineStr">
@@ -1810,11 +1810,11 @@
     </row>
     <row r="30" spans="1:14">
       <c r="A30" s="0">
-        <v>49971209</v>
+        <v>50015763</v>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>顺丰顺水</t>
+          <t>北斗星</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:29:41</t>
+          <t>2026-09-03 23:09:39</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
@@ -1870,11 +1870,11 @@
     </row>
     <row r="31" spans="1:14">
       <c r="A31" s="0">
-        <v>49970732</v>
+        <v>49989442</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>冬梅花儿开王丽君</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:13:53</t>
+          <t>2026-09-03 12:23:43</t>
         </is>
       </c>
       <c r="H31" s="0" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="I31" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J31" s="0" t="inlineStr">
@@ -1930,11 +1930,11 @@
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="0">
-        <v>49970712</v>
+        <v>49989431</v>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>月色琴弦</t>
+          <t>风声</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:13:07</t>
+          <t>2026-09-03 12:23:25</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="I32" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J32" s="0" t="inlineStr">
@@ -1990,11 +1990,11 @@
     </row>
     <row r="33" spans="1:14">
       <c r="A33" s="0">
-        <v>49970699</v>
+        <v>49989419</v>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>铜铃</t>
+          <t>胡宾</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:49</t>
+          <t>2026-09-03 12:23:13</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="I33" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J33" s="0" t="inlineStr">
@@ -2050,11 +2050,11 @@
     </row>
     <row r="34" spans="1:14">
       <c r="A34" s="0">
-        <v>49970698</v>
+        <v>49989410</v>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>东风吹</t>
+          <t>永远</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:47</t>
+          <t>2026-09-03 12:23:03</t>
         </is>
       </c>
       <c r="H34" s="0" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="I34" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J34" s="0" t="inlineStr">
@@ -2110,11 +2110,11 @@
     </row>
     <row r="35" spans="1:14">
       <c r="A35" s="0">
-        <v>49970683</v>
+        <v>49984259</v>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>杨永强</t>
+          <t>好运包张</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:17</t>
+          <t>2026-09-03 09:55:37</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J35" s="0" t="inlineStr">
@@ -2170,11 +2170,11 @@
     </row>
     <row r="36" spans="1:14">
       <c r="A36" s="0">
-        <v>49970662</v>
+        <v>49984055</v>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>盈丰</t>
+          <t>点点星辰</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:33</t>
+          <t>2026-09-03 09:49:33</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
@@ -2230,11 +2230,11 @@
     </row>
     <row r="37" spans="1:14">
       <c r="A37" s="0">
-        <v>49970652</v>
+        <v>49983134</v>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>YAN</t>
+          <t>Zhangrruzhen张如真</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -2259,7 +2259,7 @@
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:15</t>
+          <t>2026-09-03 09:25:21</t>
         </is>
       </c>
       <c r="H37" s="0" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="I37" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J37" s="0" t="inlineStr">
@@ -2290,11 +2290,11 @@
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="0">
-        <v>49970649</v>
+        <v>49971209</v>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>彩虹（宋荷娣）</t>
+          <t>顺丰顺水</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:11</t>
+          <t>2026-09-02 23:29:41</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
@@ -2350,11 +2350,11 @@
     </row>
     <row r="39" spans="1:14">
       <c r="A39" s="0">
-        <v>49970648</v>
+        <v>49970732</v>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>天知心</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:08</t>
+          <t>2026-09-02 23:13:53</t>
         </is>
       </c>
       <c r="H39" s="0" t="inlineStr">
@@ -2410,11 +2410,11 @@
     </row>
     <row r="40" spans="1:14">
       <c r="A40" s="0">
-        <v>49970643</v>
+        <v>49970712</v>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>好运来</t>
+          <t>月色琴弦</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:10:55</t>
+          <t>2026-09-02 23:13:07</t>
         </is>
       </c>
       <c r="H40" s="0" t="inlineStr">
@@ -2470,11 +2470,11 @@
     </row>
     <row r="41" spans="1:14">
       <c r="A41" s="0">
-        <v>49937566</v>
+        <v>49970699</v>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>简单sincerity</t>
+          <t>铜铃</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 10:10:33</t>
+          <t>2026-09-02 23:12:49</t>
         </is>
       </c>
       <c r="H41" s="0" t="inlineStr">
@@ -2530,11 +2530,11 @@
     </row>
     <row r="42" spans="1:14">
       <c r="A42" s="0">
-        <v>49937187</v>
+        <v>49970698</v>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>莲子</t>
+          <t>东风吹</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:58:56</t>
+          <t>2026-09-02 23:12:47</t>
         </is>
       </c>
       <c r="H42" s="0" t="inlineStr">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="I42" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J42" s="0" t="inlineStr">
@@ -2590,11 +2590,11 @@
     </row>
     <row r="43" spans="1:14">
       <c r="A43" s="0">
-        <v>49937101</v>
+        <v>49970683</v>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>蓉儿</t>
+          <t>杨永强</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:56:16</t>
+          <t>2026-09-02 23:12:17</t>
         </is>
       </c>
       <c r="H43" s="0" t="inlineStr">
@@ -2650,11 +2650,11 @@
     </row>
     <row r="44" spans="1:14">
       <c r="A44" s="0">
-        <v>49937098</v>
+        <v>49970662</v>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>瀚林2368</t>
+          <t>盈丰</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:56:15</t>
+          <t>2026-09-02 23:11:33</t>
         </is>
       </c>
       <c r="H44" s="0" t="inlineStr">
@@ -2710,11 +2710,11 @@
     </row>
     <row r="45" spans="1:14">
       <c r="A45" s="0">
-        <v>49937081</v>
+        <v>49970652</v>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>🔱 花中之美</t>
+          <t>YAN</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:47</t>
+          <t>2026-09-02 23:11:15</t>
         </is>
       </c>
       <c r="H45" s="0" t="inlineStr">
@@ -2770,11 +2770,11 @@
     </row>
     <row r="46" spans="1:14">
       <c r="A46" s="0">
-        <v>49937066</v>
+        <v>49970649</v>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>雨情</t>
+          <t>彩虹（宋荷娣）</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:27</t>
+          <t>2026-09-02 23:11:11</t>
         </is>
       </c>
       <c r="H46" s="0" t="inlineStr">
@@ -2830,11 +2830,11 @@
     </row>
     <row r="47" spans="1:14">
       <c r="A47" s="0">
-        <v>49937061</v>
+        <v>49970648</v>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>Sunny 🎈瑶</t>
+          <t>天知心</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:23</t>
+          <t>2026-09-02 23:11:08</t>
         </is>
       </c>
       <c r="H47" s="0" t="inlineStr">
@@ -2890,11 +2890,11 @@
     </row>
     <row r="48" spans="1:14">
       <c r="A48" s="0">
-        <v>49887876</v>
+        <v>49970643</v>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>鱼靖儿</t>
+          <t>好运来</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:23:11</t>
+          <t>2026-09-02 23:10:55</t>
         </is>
       </c>
       <c r="H48" s="0" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="I48" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J48" s="0" t="inlineStr">
@@ -2950,11 +2950,11 @@
     </row>
     <row r="49" spans="1:14">
       <c r="A49" s="0">
-        <v>49887478</v>
+        <v>49937566</v>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>风调雨顺</t>
+          <t>简单sincerity</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:10:17</t>
+          <t>2026-09-02 10:10:33</t>
         </is>
       </c>
       <c r="H49" s="0" t="inlineStr">
@@ -3010,11 +3010,11 @@
     </row>
     <row r="50" spans="1:14">
       <c r="A50" s="0">
-        <v>49887447</v>
+        <v>49937187</v>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>中国艺人</t>
+          <t>莲子</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:44</t>
+          <t>2026-09-02 09:58:56</t>
         </is>
       </c>
       <c r="H50" s="0" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="I50" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J50" s="0" t="inlineStr">
@@ -3070,11 +3070,11 @@
     </row>
     <row r="51" spans="1:14">
       <c r="A51" s="0">
-        <v>49887439</v>
+        <v>49937101</v>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>黄晓玲</t>
+          <t>蓉儿</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:17</t>
+          <t>2026-09-02 09:56:16</t>
         </is>
       </c>
       <c r="H51" s="0" t="inlineStr">
@@ -3130,11 +3130,11 @@
     </row>
     <row r="52" spans="1:14">
       <c r="A52" s="0">
-        <v>49887437</v>
+        <v>49937098</v>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>随缘</t>
+          <t>瀚林2368</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:07</t>
+          <t>2026-09-02 09:56:15</t>
         </is>
       </c>
       <c r="H52" s="0" t="inlineStr">
@@ -3190,11 +3190,11 @@
     </row>
     <row r="53" spans="1:14">
       <c r="A53" s="0">
-        <v>49887416</v>
+        <v>49937081</v>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>刘秋红</t>
+          <t>🔱 花中之美</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:31</t>
+          <t>2026-09-02 09:55:47</t>
         </is>
       </c>
       <c r="H53" s="0" t="inlineStr">
@@ -3250,11 +3250,11 @@
     </row>
     <row r="54" spans="1:14">
       <c r="A54" s="0">
-        <v>49887403</v>
+        <v>49937066</v>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>Mr.</t>
+          <t>雨情</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:05</t>
+          <t>2026-09-02 09:55:27</t>
         </is>
       </c>
       <c r="H54" s="0" t="inlineStr">
@@ -3310,11 +3310,11 @@
     </row>
     <row r="55" spans="1:14">
       <c r="A55" s="0">
-        <v>49887401</v>
+        <v>49937061</v>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>万事如意</t>
+          <t>Sunny 🎈瑶</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:03</t>
+          <t>2026-09-02 09:55:23</t>
         </is>
       </c>
       <c r="H55" s="0" t="inlineStr">
@@ -3370,11 +3370,11 @@
     </row>
     <row r="56" spans="1:14">
       <c r="A56" s="0">
-        <v>49887400</v>
+        <v>49887876</v>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>💋诺墨</t>
+          <t>鱼靖儿</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -3399,7 +3399,7 @@
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:01</t>
+          <t>2026-08-31 23:23:11</t>
         </is>
       </c>
       <c r="H56" s="0" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="I56" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J56" s="0" t="inlineStr">
@@ -3430,11 +3430,11 @@
     </row>
     <row r="57" spans="1:14">
       <c r="A57" s="0">
-        <v>49887399</v>
+        <v>49887478</v>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>听风</t>
+          <t>风调雨顺</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -3459,7 +3459,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:06:59</t>
+          <t>2026-08-31 23:10:17</t>
         </is>
       </c>
       <c r="H57" s="0" t="inlineStr">
@@ -3490,11 +3490,11 @@
     </row>
     <row r="58" spans="1:14">
       <c r="A58" s="0">
-        <v>49845584</v>
+        <v>49887447</v>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>彭汉平13024282926</t>
+          <t>中国艺人</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:18:55</t>
+          <t>2026-08-31 23:08:44</t>
         </is>
       </c>
       <c r="H58" s="0" t="inlineStr">
@@ -3550,11 +3550,11 @@
     </row>
     <row r="59" spans="1:14">
       <c r="A59" s="0">
-        <v>49845487</v>
+        <v>49887439</v>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>Z国华</t>
+          <t>黄晓玲</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:15:49</t>
+          <t>2026-08-31 23:08:17</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="I59" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J59" s="0" t="inlineStr">
@@ -3610,11 +3610,11 @@
     </row>
     <row r="60" spans="1:14">
       <c r="A60" s="0">
-        <v>49845407</v>
+        <v>49887437</v>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>月亮🌛</t>
+          <t>随缘</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:12:33</t>
+          <t>2026-08-31 23:08:07</t>
         </is>
       </c>
       <c r="H60" s="0" t="inlineStr">
@@ -3670,11 +3670,11 @@
     </row>
     <row r="61" spans="1:14">
       <c r="A61" s="0">
-        <v>49845398</v>
+        <v>49887416</v>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>老树</t>
+          <t>刘秋红</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:12:03</t>
+          <t>2026-08-31 23:07:31</t>
         </is>
       </c>
       <c r="H61" s="0" t="inlineStr">
@@ -3730,11 +3730,11 @@
     </row>
     <row r="62" spans="1:14">
       <c r="A62" s="0">
-        <v>49845391</v>
+        <v>49887403</v>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>八哥</t>
+          <t>Mr.</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:45</t>
+          <t>2026-08-31 23:07:05</t>
         </is>
       </c>
       <c r="H62" s="0" t="inlineStr">
@@ -3790,11 +3790,11 @@
     </row>
     <row r="63" spans="1:14">
       <c r="A63" s="0">
-        <v>49845380</v>
+        <v>49887401</v>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>铲车主出租15352562068</t>
+          <t>万事如意</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:29</t>
+          <t>2026-08-31 23:07:03</t>
         </is>
       </c>
       <c r="H63" s="0" t="inlineStr">
@@ -3850,11 +3850,11 @@
     </row>
     <row r="64" spans="1:14">
       <c r="A64" s="0">
-        <v>49845376</v>
+        <v>49887400</v>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>刘萍</t>
+          <t>💋诺墨</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:15</t>
+          <t>2026-08-31 23:07:01</t>
         </is>
       </c>
       <c r="H64" s="0" t="inlineStr">
@@ -3910,11 +3910,11 @@
     </row>
     <row r="65" spans="1:14">
       <c r="A65" s="0">
-        <v>49845374</v>
+        <v>49887399</v>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>空谷幽兰</t>
+          <t>听风</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:07</t>
+          <t>2026-08-31 23:06:59</t>
         </is>
       </c>
       <c r="H65" s="0" t="inlineStr">
@@ -3970,11 +3970,11 @@
     </row>
     <row r="66" spans="1:14">
       <c r="A66" s="0">
-        <v>49845373</v>
+        <v>49845584</v>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>泽浩羊</t>
+          <t>彭汉平13024282926</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:05</t>
+          <t>2026-08-30 23:18:55</t>
         </is>
       </c>
       <c r="H66" s="0" t="inlineStr">
@@ -4030,11 +4030,11 @@
     </row>
     <row r="67" spans="1:14">
       <c r="A67" s="0">
-        <v>49845367</v>
+        <v>49845487</v>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>峰回路转</t>
+          <t>Z国华</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:55</t>
+          <t>2026-08-30 23:15:49</t>
         </is>
       </c>
       <c r="H67" s="0" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="I67" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J67" s="0" t="inlineStr">
@@ -4090,11 +4090,11 @@
     </row>
     <row r="68" spans="1:14">
       <c r="A68" s="0">
-        <v>49845366</v>
+        <v>49845407</v>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>超儿</t>
+          <t>月亮🌛</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:51</t>
+          <t>2026-08-30 23:12:33</t>
         </is>
       </c>
       <c r="H68" s="0" t="inlineStr">
@@ -4150,11 +4150,11 @@
     </row>
     <row r="69" spans="1:14">
       <c r="A69" s="0">
-        <v>49845365</v>
+        <v>49845398</v>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>传</t>
+          <t>老树</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:49</t>
+          <t>2026-08-30 23:12:03</t>
         </is>
       </c>
       <c r="H69" s="0" t="inlineStr">
@@ -4210,11 +4210,11 @@
     </row>
     <row r="70" spans="1:14">
       <c r="A70" s="0">
-        <v>49845360</v>
+        <v>49845391</v>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>悟歌</t>
+          <t>八哥</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:43</t>
+          <t>2026-08-30 23:11:45</t>
         </is>
       </c>
       <c r="H70" s="0" t="inlineStr">
@@ -4270,11 +4270,11 @@
     </row>
     <row r="71" spans="1:14">
       <c r="A71" s="0">
-        <v>49845342</v>
+        <v>49845380</v>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>丽丽</t>
+          <t>铲车主出租15352562068</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -4299,7 +4299,7 @@
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:15</t>
+          <t>2026-08-30 23:11:29</t>
         </is>
       </c>
       <c r="H71" s="0" t="inlineStr">
@@ -4330,11 +4330,11 @@
     </row>
     <row r="72" spans="1:14">
       <c r="A72" s="0">
-        <v>49826011</v>
+        <v>49845376</v>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>王前卫</t>
+          <t>刘萍</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:57:27</t>
+          <t>2026-08-30 23:11:15</t>
         </is>
       </c>
       <c r="H72" s="0" t="inlineStr">
@@ -4390,11 +4390,11 @@
     </row>
     <row r="73" spans="1:14">
       <c r="A73" s="0">
-        <v>49825720</v>
+        <v>49845374</v>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>老A</t>
+          <t>空谷幽兰</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:46:02</t>
+          <t>2026-08-30 23:11:07</t>
         </is>
       </c>
       <c r="H73" s="0" t="inlineStr">
@@ -4450,11 +4450,11 @@
     </row>
     <row r="74" spans="1:14">
       <c r="A74" s="0">
-        <v>49825676</v>
+        <v>49845373</v>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>蓝天</t>
+          <t>泽浩羊</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:44:05</t>
+          <t>2026-08-30 23:11:05</t>
         </is>
       </c>
       <c r="H74" s="0" t="inlineStr">
@@ -4510,11 +4510,11 @@
     </row>
     <row r="75" spans="1:14">
       <c r="A75" s="0">
-        <v>49825650</v>
+        <v>49845367</v>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>爱芳</t>
+          <t>峰回路转</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -4539,7 +4539,7 @@
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:43:11</t>
+          <t>2026-08-30 23:10:55</t>
         </is>
       </c>
       <c r="H75" s="0" t="inlineStr">
@@ -4570,11 +4570,11 @@
     </row>
     <row r="76" spans="1:14">
       <c r="A76" s="0">
-        <v>49825642</v>
+        <v>49845366</v>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>银杏树</t>
+          <t>超儿</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -4599,7 +4599,7 @@
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:55</t>
+          <t>2026-08-30 23:10:51</t>
         </is>
       </c>
       <c r="H76" s="0" t="inlineStr">
@@ -4630,11 +4630,11 @@
     </row>
     <row r="77" spans="1:14">
       <c r="A77" s="0">
-        <v>49825640</v>
+        <v>49845365</v>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>遵命有福（杨凤）</t>
+          <t>传</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:49</t>
+          <t>2026-08-30 23:10:49</t>
         </is>
       </c>
       <c r="H77" s="0" t="inlineStr">
@@ -4690,11 +4690,11 @@
     </row>
     <row r="78" spans="1:14">
       <c r="A78" s="0">
-        <v>49825639</v>
+        <v>49845360</v>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>申华</t>
+          <t>悟歌</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -4719,7 +4719,7 @@
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:49</t>
+          <t>2026-08-30 23:10:43</t>
         </is>
       </c>
       <c r="H78" s="0" t="inlineStr">
@@ -4750,11 +4750,11 @@
     </row>
     <row r="79" spans="1:14">
       <c r="A79" s="0">
-        <v>49825637</v>
+        <v>49845342</v>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>陈月焓</t>
+          <t>丽丽</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -4779,7 +4779,7 @@
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:47</t>
+          <t>2026-08-30 23:10:15</t>
         </is>
       </c>
       <c r="H79" s="0" t="inlineStr">
@@ -4810,11 +4810,11 @@
     </row>
     <row r="80" spans="1:14">
       <c r="A80" s="0">
-        <v>49825635</v>
+        <v>49826011</v>
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>小镇生活&amp;&amp;杜震</t>
+          <t>王前卫</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:43</t>
+          <t>2026-08-30 12:57:27</t>
         </is>
       </c>
       <c r="H80" s="0" t="inlineStr">
@@ -4870,11 +4870,11 @@
     </row>
     <row r="81" spans="1:14">
       <c r="A81" s="0">
-        <v>49825628</v>
+        <v>49825720</v>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>Taᴗaoᥫᩣ</t>
+          <t>老A</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:35</t>
+          <t>2026-08-30 12:46:02</t>
         </is>
       </c>
       <c r="H81" s="0" t="inlineStr">
@@ -4930,11 +4930,11 @@
     </row>
     <row r="82" spans="1:14">
       <c r="A82" s="0">
-        <v>49782066</v>
+        <v>49825676</v>
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>前程似锦</t>
+          <t>蓝天</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 09:07:29</t>
+          <t>2026-08-30 12:44:05</t>
         </is>
       </c>
       <c r="H82" s="0" t="inlineStr">
@@ -4969,7 +4969,7 @@
       </c>
       <c r="I82" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J82" s="0" t="inlineStr">
@@ -4990,11 +4990,11 @@
     </row>
     <row r="83" spans="1:14">
       <c r="A83" s="0">
-        <v>49771027</v>
+        <v>49825650</v>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>非比</t>
+          <t>爱芳</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -5019,7 +5019,7 @@
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 23:30:09</t>
+          <t>2026-08-30 12:43:11</t>
         </is>
       </c>
       <c r="H83" s="0" t="inlineStr">
@@ -5029,7 +5029,7 @@
       </c>
       <c r="I83" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J83" s="0" t="inlineStr">
@@ -5050,11 +5050,11 @@
     </row>
     <row r="84" spans="1:14">
       <c r="A84" s="0">
-        <v>49673360</v>
+        <v>49825642</v>
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>德行天下</t>
+          <t>银杏树</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:19:03</t>
+          <t>2026-08-30 12:42:55</t>
         </is>
       </c>
       <c r="H84" s="0" t="inlineStr">
@@ -5089,7 +5089,7 @@
       </c>
       <c r="I84" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J84" s="0" t="inlineStr">
@@ -5110,11 +5110,11 @@
     </row>
     <row r="85" spans="1:14">
       <c r="A85" s="0">
-        <v>49673352</v>
+        <v>49825640</v>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>余盛将至2026</t>
+          <t>遵命有福（杨凤）</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:49</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H85" s="0" t="inlineStr">
@@ -5149,7 +5149,7 @@
       </c>
       <c r="I85" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J85" s="0" t="inlineStr">
@@ -5170,11 +5170,11 @@
     </row>
     <row r="86" spans="1:14">
       <c r="A86" s="0">
-        <v>49673350</v>
+        <v>49825639</v>
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>山居客</t>
+          <t>申华</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -5199,7 +5199,7 @@
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:47</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H86" s="0" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="I86" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J86" s="0" t="inlineStr">
@@ -5230,11 +5230,11 @@
     </row>
     <row r="87" spans="1:14">
       <c r="A87" s="0">
-        <v>49673349</v>
+        <v>49825637</v>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>白云</t>
+          <t>陈月焓</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:45</t>
+          <t>2026-08-30 12:42:47</t>
         </is>
       </c>
       <c r="H87" s="0" t="inlineStr">
@@ -5269,7 +5269,7 @@
       </c>
       <c r="I87" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J87" s="0" t="inlineStr">
@@ -5290,11 +5290,11 @@
     </row>
     <row r="88" spans="1:14">
       <c r="A88" s="0">
-        <v>49646935</v>
+        <v>49825635</v>
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>马跃荣</t>
+          <t>小镇生活&amp;&amp;杜震</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -5319,7 +5319,7 @@
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:59</t>
+          <t>2026-08-30 12:42:43</t>
         </is>
       </c>
       <c r="H88" s="0" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="I88" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J88" s="0" t="inlineStr">
@@ -5350,11 +5350,11 @@
     </row>
     <row r="89" spans="1:14">
       <c r="A89" s="0">
-        <v>49646933</v>
+        <v>49825628</v>
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>@吴</t>
+          <t>Taᴗaoᥫᩣ</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:56</t>
+          <t>2026-08-30 12:42:35</t>
         </is>
       </c>
       <c r="H89" s="0" t="inlineStr">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="I89" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J89" s="0" t="inlineStr">
@@ -5410,11 +5410,11 @@
     </row>
     <row r="90" spans="1:14">
       <c r="A90" s="0">
-        <v>49646901</v>
+        <v>49782066</v>
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>龙安：富华／</t>
+          <t>前程似锦</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:14:28</t>
+          <t>2026-08-29 09:07:29</t>
         </is>
       </c>
       <c r="H90" s="0" t="inlineStr">
@@ -5449,7 +5449,7 @@
       </c>
       <c r="I90" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J90" s="0" t="inlineStr">
@@ -5470,11 +5470,11 @@
     </row>
     <row r="91" spans="1:14">
       <c r="A91" s="0">
-        <v>49646876</v>
+        <v>49771027</v>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>冬日暖阳🌻</t>
+          <t>非比</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:37</t>
+          <t>2026-08-28 23:30:09</t>
         </is>
       </c>
       <c r="H91" s="0" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="I91" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J91" s="0" t="inlineStr">
@@ -5530,11 +5530,11 @@
     </row>
     <row r="92" spans="1:14">
       <c r="A92" s="0">
-        <v>49646867</v>
+        <v>49673360</v>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t>寒雨</t>
+          <t>德行天下</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="G92" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:15</t>
+          <t>2026-08-26 12:19:03</t>
         </is>
       </c>
       <c r="H92" s="0" t="inlineStr">
@@ -5590,11 +5590,11 @@
     </row>
     <row r="93" spans="1:14">
       <c r="A93" s="0">
-        <v>49636232</v>
+        <v>49673352</v>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t>平安</t>
+          <t>余盛将至2026</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:20:15</t>
+          <t>2026-08-26 12:18:49</t>
         </is>
       </c>
       <c r="H93" s="0" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="I93" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J93" s="0" t="inlineStr">
@@ -5650,11 +5650,11 @@
     </row>
     <row r="94" spans="1:14">
       <c r="A94" s="0">
-        <v>49636184</v>
+        <v>49673350</v>
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t>古道西风</t>
+          <t>山居客</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
@@ -5679,7 +5679,7 @@
       </c>
       <c r="G94" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:55</t>
+          <t>2026-08-26 12:18:47</t>
         </is>
       </c>
       <c r="H94" s="0" t="inlineStr">
@@ -5689,7 +5689,7 @@
       </c>
       <c r="I94" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J94" s="0" t="inlineStr">
@@ -5710,11 +5710,11 @@
     </row>
     <row r="95" spans="1:14">
       <c r="A95" s="0">
-        <v>49636170</v>
+        <v>49673349</v>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>周海龙</t>
+          <t>白云</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="G95" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:33</t>
+          <t>2026-08-26 12:18:45</t>
         </is>
       </c>
       <c r="H95" s="0" t="inlineStr">
@@ -5749,7 +5749,7 @@
       </c>
       <c r="I95" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J95" s="0" t="inlineStr">
@@ -5770,11 +5770,11 @@
     </row>
     <row r="96" spans="1:14">
       <c r="A96" s="0">
-        <v>49636157</v>
+        <v>49646935</v>
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t>锦妍</t>
+          <t>马跃荣</t>
         </is>
       </c>
       <c r="C96" s="0" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="G96" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:07</t>
+          <t>2026-08-25 18:15:59</t>
         </is>
       </c>
       <c r="H96" s="0" t="inlineStr">
@@ -5809,7 +5809,7 @@
       </c>
       <c r="I96" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J96" s="0" t="inlineStr">
@@ -5830,11 +5830,11 @@
     </row>
     <row r="97" spans="1:14">
       <c r="A97" s="0">
-        <v>49593974</v>
+        <v>49646933</v>
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>兰兰</t>
+          <t>@吴</t>
         </is>
       </c>
       <c r="C97" s="0" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="G97" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:59:53</t>
+          <t>2026-08-25 18:15:56</t>
         </is>
       </c>
       <c r="H97" s="0" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="I97" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J97" s="0" t="inlineStr">
@@ -5890,11 +5890,11 @@
     </row>
     <row r="98" spans="1:14">
       <c r="A98" s="0">
-        <v>49593671</v>
+        <v>49646901</v>
       </c>
       <c r="B98" s="0" t="inlineStr">
         <is>
-          <t>准备1号</t>
+          <t>龙安：富华／</t>
         </is>
       </c>
       <c r="C98" s="0" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="G98" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:49:27</t>
+          <t>2026-08-25 18:14:28</t>
         </is>
       </c>
       <c r="H98" s="0" t="inlineStr">
@@ -5929,7 +5929,7 @@
       </c>
       <c r="I98" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J98" s="0" t="inlineStr">
@@ -5950,11 +5950,11 @@
     </row>
     <row r="99" spans="1:14">
       <c r="A99" s="0">
-        <v>49535916</v>
+        <v>49646876</v>
       </c>
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t>真诚</t>
+          <t>冬日暖阳🌻</t>
         </is>
       </c>
       <c r="C99" s="0" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="G99" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:46:23</t>
+          <t>2026-08-25 18:13:37</t>
         </is>
       </c>
       <c r="H99" s="0" t="inlineStr">
@@ -5989,7 +5989,7 @@
       </c>
       <c r="I99" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J99" s="0" t="inlineStr">
@@ -6010,11 +6010,11 @@
     </row>
     <row r="100" spans="1:14">
       <c r="A100" s="0">
-        <v>49535653</v>
+        <v>49646867</v>
       </c>
       <c r="B100" s="0" t="inlineStr">
         <is>
-          <t>如意家电13368134456维修</t>
+          <t>寒雨</t>
         </is>
       </c>
       <c r="C100" s="0" t="inlineStr">
@@ -6039,7 +6039,7 @@
       </c>
       <c r="G100" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:28:25</t>
+          <t>2026-08-25 18:13:15</t>
         </is>
       </c>
       <c r="H100" s="0" t="inlineStr">
@@ -6049,7 +6049,7 @@
       </c>
       <c r="I100" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J100" s="0" t="inlineStr">
@@ -6070,11 +6070,11 @@
     </row>
     <row r="101" spans="1:14">
       <c r="A101" s="0">
-        <v>49535650</v>
+        <v>49636232</v>
       </c>
       <c r="B101" s="0" t="inlineStr">
         <is>
-          <t>莺莺</t>
+          <t>平安</t>
         </is>
       </c>
       <c r="C101" s="0" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="G101" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:27:55</t>
+          <t>2026-08-25 13:20:15</t>
         </is>
       </c>
       <c r="H101" s="0" t="inlineStr">
@@ -6125,21 +6125,16 @@
       <c r="L101" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N101" s="0" t="inlineStr">
-        <is>
-          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="102" spans="1:14">
       <c r="A102" s="0">
-        <v>49508265</v>
+        <v>49636184</v>
       </c>
       <c r="B102" s="0" t="inlineStr">
         <is>
-          <t>爱猫🐱 咪</t>
+          <t>古道西风</t>
         </is>
       </c>
       <c r="C102" s="0" t="inlineStr">
@@ -6164,7 +6159,7 @@
       </c>
       <c r="G102" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 09:53:41</t>
+          <t>2026-08-25 13:18:55</t>
         </is>
       </c>
       <c r="H102" s="0" t="inlineStr">
@@ -6174,7 +6169,7 @@
       </c>
       <c r="I102" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J102" s="0" t="inlineStr">
@@ -6195,11 +6190,11 @@
     </row>
     <row r="103" spans="1:14">
       <c r="A103" s="0">
-        <v>49493414</v>
+        <v>49636170</v>
       </c>
       <c r="B103" s="0" t="inlineStr">
         <is>
-          <t>惠平</t>
+          <t>周海龙</t>
         </is>
       </c>
       <c r="C103" s="0" t="inlineStr">
@@ -6224,7 +6219,7 @@
       </c>
       <c r="G103" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:53:02</t>
+          <t>2026-08-25 13:18:33</t>
         </is>
       </c>
       <c r="H103" s="0" t="inlineStr">
@@ -6234,7 +6229,7 @@
       </c>
       <c r="I103" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J103" s="0" t="inlineStr">
@@ -6255,11 +6250,11 @@
     </row>
     <row r="104" spans="1:14">
       <c r="A104" s="0">
-        <v>49493126</v>
+        <v>49636157</v>
       </c>
       <c r="B104" s="0" t="inlineStr">
         <is>
-          <t>刘盼昭</t>
+          <t>锦妍</t>
         </is>
       </c>
       <c r="C104" s="0" t="inlineStr">
@@ -6284,7 +6279,7 @@
       </c>
       <c r="G104" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:44:53</t>
+          <t>2026-08-25 13:18:07</t>
         </is>
       </c>
       <c r="H104" s="0" t="inlineStr">
@@ -6294,7 +6289,7 @@
       </c>
       <c r="I104" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J104" s="0" t="inlineStr">
@@ -6315,11 +6310,11 @@
     </row>
     <row r="105" spans="1:14">
       <c r="A105" s="0">
-        <v>49492499</v>
+        <v>49593974</v>
       </c>
       <c r="B105" s="0" t="inlineStr">
         <is>
-          <t>红霞</t>
+          <t>兰兰</t>
         </is>
       </c>
       <c r="C105" s="0" t="inlineStr">
@@ -6344,7 +6339,7 @@
       </c>
       <c r="G105" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:29:43</t>
+          <t>2026-08-24 12:59:53</t>
         </is>
       </c>
       <c r="H105" s="0" t="inlineStr">
@@ -6375,11 +6370,11 @@
     </row>
     <row r="106" spans="1:14">
       <c r="A106" s="0">
-        <v>49455301</v>
+        <v>49593671</v>
       </c>
       <c r="B106" s="0" t="inlineStr">
         <is>
-          <t>周开平</t>
+          <t>准备1号</t>
         </is>
       </c>
       <c r="C106" s="0" t="inlineStr">
@@ -6404,7 +6399,7 @@
       </c>
       <c r="G106" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 22:46:59</t>
+          <t>2026-08-24 12:49:27</t>
         </is>
       </c>
       <c r="H106" s="0" t="inlineStr">
@@ -6435,11 +6430,11 @@
     </row>
     <row r="107" spans="1:14">
       <c r="A107" s="0">
-        <v>49432023</v>
+        <v>49535916</v>
       </c>
       <c r="B107" s="0" t="inlineStr">
         <is>
-          <t>花生米</t>
+          <t>真诚</t>
         </is>
       </c>
       <c r="C107" s="0" t="inlineStr">
@@ -6464,7 +6459,7 @@
       </c>
       <c r="G107" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 11:55:45</t>
+          <t>2026-08-22 23:46:23</t>
         </is>
       </c>
       <c r="H107" s="0" t="inlineStr">
@@ -6495,11 +6490,11 @@
     </row>
     <row r="108" spans="1:14">
       <c r="A108" s="0">
-        <v>49415939</v>
+        <v>49535653</v>
       </c>
       <c r="B108" s="0" t="inlineStr">
         <is>
-          <t>杨梅芳</t>
+          <t>如意家电13368134456维修</t>
         </is>
       </c>
       <c r="C108" s="0" t="inlineStr">
@@ -6524,7 +6519,7 @@
       </c>
       <c r="G108" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:58</t>
+          <t>2026-08-22 23:28:25</t>
         </is>
       </c>
       <c r="H108" s="0" t="inlineStr">
@@ -6534,17 +6529,17 @@
       </c>
       <c r="I108" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J108" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K108" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L108" s="0" t="inlineStr">
@@ -6555,11 +6550,11 @@
     </row>
     <row r="109" spans="1:14">
       <c r="A109" s="0">
-        <v>49415918</v>
+        <v>49535650</v>
       </c>
       <c r="B109" s="0" t="inlineStr">
         <is>
-          <t>心语无言</t>
+          <t>莺莺</t>
         </is>
       </c>
       <c r="C109" s="0" t="inlineStr">
@@ -6584,7 +6579,7 @@
       </c>
       <c r="G109" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:24</t>
+          <t>2026-08-22 23:27:55</t>
         </is>
       </c>
       <c r="H109" s="0" t="inlineStr">
@@ -6594,32 +6589,37 @@
       </c>
       <c r="I109" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J109" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K109" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L109" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N109" s="0" t="inlineStr">
+        <is>
+          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="110" spans="1:14">
       <c r="A110" s="0">
-        <v>49415913</v>
+        <v>49508265</v>
       </c>
       <c r="B110" s="0" t="inlineStr">
         <is>
-          <t>安好</t>
+          <t>爱猫🐱 咪</t>
         </is>
       </c>
       <c r="C110" s="0" t="inlineStr">
@@ -6644,7 +6644,7 @@
       </c>
       <c r="G110" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:18</t>
+          <t>2026-08-22 09:53:41</t>
         </is>
       </c>
       <c r="H110" s="0" t="inlineStr">
@@ -6654,17 +6654,17 @@
       </c>
       <c r="I110" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J110" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K110" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L110" s="0" t="inlineStr">
@@ -6675,11 +6675,11 @@
     </row>
     <row r="111" spans="1:14">
       <c r="A111" s="0">
-        <v>49415890</v>
+        <v>49493414</v>
       </c>
       <c r="B111" s="0" t="inlineStr">
         <is>
-          <t>雨夜聆风</t>
+          <t>惠平</t>
         </is>
       </c>
       <c r="C111" s="0" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="G111" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:56</t>
+          <t>2026-08-21 22:53:02</t>
         </is>
       </c>
       <c r="H111" s="0" t="inlineStr">
@@ -6714,37 +6714,32 @@
       </c>
       <c r="I111" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J111" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K111" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L111" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N111" s="0" t="inlineStr">
-        <is>
-          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="112" spans="1:14">
       <c r="A112" s="0">
-        <v>49415874</v>
+        <v>49493126</v>
       </c>
       <c r="B112" s="0" t="inlineStr">
         <is>
-          <t>飘</t>
+          <t>刘盼昭</t>
         </is>
       </c>
       <c r="C112" s="0" t="inlineStr">
@@ -6769,7 +6764,7 @@
       </c>
       <c r="G112" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:40</t>
+          <t>2026-08-21 22:44:53</t>
         </is>
       </c>
       <c r="H112" s="0" t="inlineStr">
@@ -6779,17 +6774,17 @@
       </c>
       <c r="I112" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J112" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K112" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L112" s="0" t="inlineStr">
@@ -6800,11 +6795,11 @@
     </row>
     <row r="113" spans="1:14">
       <c r="A113" s="0">
-        <v>49415871</v>
+        <v>49492499</v>
       </c>
       <c r="B113" s="0" t="inlineStr">
         <is>
-          <t>庆</t>
+          <t>红霞</t>
         </is>
       </c>
       <c r="C113" s="0" t="inlineStr">
@@ -6829,7 +6824,7 @@
       </c>
       <c r="G113" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:36</t>
+          <t>2026-08-21 22:29:43</t>
         </is>
       </c>
       <c r="H113" s="0" t="inlineStr">
@@ -6839,17 +6834,17 @@
       </c>
       <c r="I113" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J113" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K113" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L113" s="0" t="inlineStr">
@@ -6860,59 +6855,544 @@
     </row>
     <row r="114" spans="1:14">
       <c r="A114" s="0">
+        <v>49455301</v>
+      </c>
+      <c r="B114" s="0" t="inlineStr">
+        <is>
+          <t>周开平</t>
+        </is>
+      </c>
+      <c r="C114" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D114" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E114" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F114" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G114" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-20 22:46:59</t>
+        </is>
+      </c>
+      <c r="H114" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I114" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J114" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K114" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L114" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" spans="1:14">
+      <c r="A115" s="0">
+        <v>49432023</v>
+      </c>
+      <c r="B115" s="0" t="inlineStr">
+        <is>
+          <t>花生米</t>
+        </is>
+      </c>
+      <c r="C115" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D115" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E115" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F115" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G115" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-20 11:55:45</t>
+        </is>
+      </c>
+      <c r="H115" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I115" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J115" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K115" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L115" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" spans="1:14">
+      <c r="A116" s="0">
+        <v>49415939</v>
+      </c>
+      <c r="B116" s="0" t="inlineStr">
+        <is>
+          <t>杨梅芳</t>
+        </is>
+      </c>
+      <c r="C116" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D116" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E116" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F116" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G116" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:58</t>
+        </is>
+      </c>
+      <c r="H116" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I116" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J116" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K116" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L116" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" spans="1:14">
+      <c r="A117" s="0">
+        <v>49415918</v>
+      </c>
+      <c r="B117" s="0" t="inlineStr">
+        <is>
+          <t>心语无言</t>
+        </is>
+      </c>
+      <c r="C117" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D117" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E117" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F117" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G117" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:24</t>
+        </is>
+      </c>
+      <c r="H117" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I117" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J117" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K117" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L117" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" spans="1:14">
+      <c r="A118" s="0">
+        <v>49415913</v>
+      </c>
+      <c r="B118" s="0" t="inlineStr">
+        <is>
+          <t>安好</t>
+        </is>
+      </c>
+      <c r="C118" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D118" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E118" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F118" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G118" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:18</t>
+        </is>
+      </c>
+      <c r="H118" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I118" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J118" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K118" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L118" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" spans="1:14">
+      <c r="A119" s="0">
+        <v>49415890</v>
+      </c>
+      <c r="B119" s="0" t="inlineStr">
+        <is>
+          <t>雨夜聆风</t>
+        </is>
+      </c>
+      <c r="C119" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D119" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E119" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F119" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G119" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:56</t>
+        </is>
+      </c>
+      <c r="H119" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I119" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J119" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K119" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L119" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="N119" s="0" t="inlineStr">
+        <is>
+          <t>宜春</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" spans="1:14">
+      <c r="A120" s="0">
+        <v>49415874</v>
+      </c>
+      <c r="B120" s="0" t="inlineStr">
+        <is>
+          <t>飘</t>
+        </is>
+      </c>
+      <c r="C120" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D120" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E120" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F120" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G120" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:40</t>
+        </is>
+      </c>
+      <c r="H120" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I120" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J120" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K120" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L120" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" spans="1:14">
+      <c r="A121" s="0">
+        <v>49415871</v>
+      </c>
+      <c r="B121" s="0" t="inlineStr">
+        <is>
+          <t>庆</t>
+        </is>
+      </c>
+      <c r="C121" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D121" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E121" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F121" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G121" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:36</t>
+        </is>
+      </c>
+      <c r="H121" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I121" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J121" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K121" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L121" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" spans="1:14">
+      <c r="A122" s="0">
         <v>49415867</v>
       </c>
-      <c r="B114" s="0" t="inlineStr">
+      <c r="B122" s="0" t="inlineStr">
         <is>
           <t>HYQ</t>
         </is>
       </c>
-      <c r="C114" s="0" t="inlineStr">
-        <is>
-          <t>6天0基础钢琴入门课</t>
-        </is>
-      </c>
-      <c r="D114" s="0" t="inlineStr">
-        <is>
-          <t>训练营</t>
-        </is>
-      </c>
-      <c r="E114" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="F114" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="G114" s="0" t="inlineStr">
+      <c r="C122" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D122" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E122" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F122" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G122" s="0" t="inlineStr">
         <is>
           <t>2026-08-19 22:47:33</t>
         </is>
       </c>
-      <c r="H114" s="0" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I114" s="0" t="inlineStr">
-        <is>
-          <t>黄老师-抖音01</t>
-        </is>
-      </c>
-      <c r="J114" s="0" t="inlineStr">
+      <c r="H122" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I122" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J122" s="0" t="inlineStr">
         <is>
           <t>安迪钢琴-多个点击报名-0元</t>
         </is>
       </c>
-      <c r="K114" s="0" t="inlineStr">
+      <c r="K122" s="0" t="inlineStr">
         <is>
           <t>微信支付</t>
         </is>
       </c>
-      <c r="L114" s="0" t="inlineStr">
+      <c r="L122" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>

</xml_diff>

<commit_message>
📅 日报更新 2026-09-05 07:06
</commit_message>
<xml_diff>
--- a/data/exports/黄老师/dist_order_2026-09-05.xlsx
+++ b/data/exports/黄老师/dist_order_2026-09-05.xlsx
@@ -125,11 +125,11 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="0">
-        <v>50074867</v>
+        <v>50080657</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>美好人生</t>
+          <t>平红</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 10:19:59</t>
+          <t>2026-09-05 13:07:13</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -164,7 +164,7 @@
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J2" s="0" t="inlineStr">
@@ -185,11 +185,11 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="0">
-        <v>50074273</v>
+        <v>50080582</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>周利平</t>
+          <t>aabb</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -214,7 +214,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 10:02:26</t>
+          <t>2026-09-05 13:05:19</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -245,11 +245,11 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="0">
-        <v>50074103</v>
+        <v>50080559</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>赵香荣</t>
+          <t>自由人</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -274,7 +274,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:58:29</t>
+          <t>2026-09-05 13:04:28</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -305,11 +305,11 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="0">
-        <v>50074078</v>
+        <v>50080553</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>长风渡℡明</t>
+          <t>晶晶</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -334,7 +334,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:49</t>
+          <t>2026-09-05 13:04:15</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -365,11 +365,11 @@
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="0">
-        <v>50074077</v>
+        <v>50080549</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>海阔天空bi</t>
+          <t>abc</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -394,7 +394,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:47</t>
+          <t>2026-09-05 13:04:09</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -425,11 +425,11 @@
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="0">
-        <v>50074076</v>
+        <v>50080548</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>枫叶红</t>
+          <t>盘子</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:47</t>
+          <t>2026-09-05 13:04:08</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -485,11 +485,11 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="0">
-        <v>50074071</v>
+        <v>50080547</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>思缘</t>
+          <t>赵满珍C5</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:35</t>
+          <t>2026-09-05 13:04:05</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -545,11 +545,11 @@
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="0">
-        <v>50074067</v>
+        <v>50080539</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>悠然</t>
+          <t>平平安安</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:25</t>
+          <t>2026-09-05 13:03:51</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -605,11 +605,11 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="0">
-        <v>50058017</v>
+        <v>50080538</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>索描贾师＃壹皇贰金山玉旗🇨🇳</t>
+          <t>凡事包容</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:16:49</t>
+          <t>2026-09-05 13:03:51</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
@@ -665,11 +665,11 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="0">
-        <v>50057895</v>
+        <v>50080536</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>南雪</t>
+          <t>吴忧无忧</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:12:32</t>
+          <t>2026-09-05 13:03:47</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -720,21 +720,16 @@
       <c r="L11" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N11" s="0" t="inlineStr">
-        <is>
-          <t>镇江</t>
         </is>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="0">
-        <v>50057857</v>
+        <v>50080535</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>可心</t>
+          <t>小鱼儿</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -759,7 +754,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:55</t>
+          <t>2026-09-05 13:03:43</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -790,11 +785,11 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="0">
-        <v>50057854</v>
+        <v>50080525</v>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>张苏龙</t>
+          <t>辞芝锦😎</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -819,7 +814,7 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:51</t>
+          <t>2026-09-05 13:03:29</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
@@ -850,11 +845,11 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="0">
-        <v>50057852</v>
+        <v>50080523</v>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>？</t>
+          <t>早陈</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -879,7 +874,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:43</t>
+          <t>2026-09-05 13:03:21</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -910,11 +905,11 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="0">
-        <v>50057841</v>
+        <v>50080516</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>向往的生活-电信号</t>
+          <t>星星の恋人</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -939,7 +934,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:09</t>
+          <t>2026-09-05 13:03:13</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -970,11 +965,11 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="0">
-        <v>50057839</v>
+        <v>50080511</v>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>金盏花</t>
+          <t>无咎</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -999,7 +994,7 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:03</t>
+          <t>2026-09-05 13:03:09</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
@@ -1030,11 +1025,11 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="0">
-        <v>50032697</v>
+        <v>50080477</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>小米. ᩚ</t>
+          <t>刘小虎</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1059,7 +1054,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:24:13</t>
+          <t>2026-09-05 13:02:37</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
@@ -1069,7 +1064,7 @@
       </c>
       <c r="I17" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J17" s="0" t="inlineStr">
@@ -1090,11 +1085,11 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="0">
-        <v>50032693</v>
+        <v>50074867</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>海岸</t>
+          <t>美好人生</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -1119,7 +1114,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:24:11</t>
+          <t>2026-09-05 10:19:59</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
@@ -1129,7 +1124,7 @@
       </c>
       <c r="I18" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J18" s="0" t="inlineStr">
@@ -1150,11 +1145,11 @@
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="0">
-        <v>50032683</v>
+        <v>50074273</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>陆建军</t>
+          <t>周利平</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -1179,7 +1174,7 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:23:53</t>
+          <t>2026-09-05 10:02:26</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
@@ -1189,7 +1184,7 @@
       </c>
       <c r="I19" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J19" s="0" t="inlineStr">
@@ -1210,11 +1205,11 @@
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="0">
-        <v>50015883</v>
+        <v>50074103</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>A00金华义乌叉车出租电15268650979</t>
+          <t>赵香荣</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -1239,7 +1234,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:18:02</t>
+          <t>2026-09-05 09:58:29</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
@@ -1249,7 +1244,7 @@
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J20" s="0" t="inlineStr">
@@ -1270,11 +1265,11 @@
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="0">
-        <v>50015882</v>
+        <v>50074078</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>建程仓储中心 张川</t>
+          <t>长风渡℡明</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -1299,7 +1294,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:18:02</t>
+          <t>2026-09-05 09:57:49</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
@@ -1330,11 +1325,11 @@
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="0">
-        <v>50015784</v>
+        <v>50074077</v>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>天空</t>
+          <t>海阔天空bi</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -1359,7 +1354,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:41</t>
+          <t>2026-09-05 09:57:47</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
@@ -1390,11 +1385,11 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="0">
-        <v>50015778</v>
+        <v>50074076</v>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>小龙女</t>
+          <t>枫叶红</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -1419,7 +1414,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:21</t>
+          <t>2026-09-05 09:57:47</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
@@ -1450,11 +1445,11 @@
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="0">
-        <v>50015776</v>
+        <v>50074071</v>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>桥梁</t>
+          <t>思缘</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -1479,7 +1474,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:15</t>
+          <t>2026-09-05 09:57:35</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -1510,11 +1505,11 @@
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="0">
-        <v>50015775</v>
+        <v>50074067</v>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>彩云之南</t>
+          <t>悠然</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -1539,7 +1534,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:13</t>
+          <t>2026-09-05 09:57:25</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
@@ -1570,11 +1565,11 @@
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="0">
-        <v>50015774</v>
+        <v>50058017</v>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>楊精蓄銳༒</t>
+          <t>索描贾师＃壹皇贰金山玉旗🇨🇳</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -1599,7 +1594,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:11</t>
+          <t>2026-09-04 23:16:49</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -1630,11 +1625,11 @@
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="0">
-        <v>50015772</v>
+        <v>50057895</v>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>不倒翁</t>
+          <t>南雪</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1659,7 +1654,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:07</t>
+          <t>2026-09-04 23:12:32</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
@@ -1685,16 +1680,21 @@
       <c r="L27" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N27" s="0" t="inlineStr">
+        <is>
+          <t>镇江</t>
         </is>
       </c>
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="0">
-        <v>50015770</v>
+        <v>50057857</v>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>一江春水</t>
+          <t>可心</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:05</t>
+          <t>2026-09-04 23:10:55</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
@@ -1750,11 +1750,11 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" s="0">
-        <v>50015767</v>
+        <v>50057854</v>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>微笑</t>
+          <t>张苏龙</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:03</t>
+          <t>2026-09-04 23:10:51</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
@@ -1810,11 +1810,11 @@
     </row>
     <row r="30" spans="1:14">
       <c r="A30" s="0">
-        <v>50015763</v>
+        <v>50057852</v>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>北斗星</t>
+          <t>？</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:09:39</t>
+          <t>2026-09-04 23:10:43</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
@@ -1870,11 +1870,11 @@
     </row>
     <row r="31" spans="1:14">
       <c r="A31" s="0">
-        <v>49989442</v>
+        <v>50057841</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>冬梅花儿开王丽君</t>
+          <t>向往的生活-电信号</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:43</t>
+          <t>2026-09-04 23:10:09</t>
         </is>
       </c>
       <c r="H31" s="0" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="I31" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J31" s="0" t="inlineStr">
@@ -1930,11 +1930,11 @@
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="0">
-        <v>49989431</v>
+        <v>50057839</v>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>风声</t>
+          <t>金盏花</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:25</t>
+          <t>2026-09-04 23:10:03</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="I32" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J32" s="0" t="inlineStr">
@@ -1990,11 +1990,11 @@
     </row>
     <row r="33" spans="1:14">
       <c r="A33" s="0">
-        <v>49989419</v>
+        <v>50032697</v>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>胡宾</t>
+          <t>小米. ᩚ</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:13</t>
+          <t>2026-09-04 12:24:13</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
@@ -2050,11 +2050,11 @@
     </row>
     <row r="34" spans="1:14">
       <c r="A34" s="0">
-        <v>49989410</v>
+        <v>50032693</v>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>永远</t>
+          <t>海岸</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:03</t>
+          <t>2026-09-04 12:24:11</t>
         </is>
       </c>
       <c r="H34" s="0" t="inlineStr">
@@ -2110,11 +2110,11 @@
     </row>
     <row r="35" spans="1:14">
       <c r="A35" s="0">
-        <v>49984259</v>
+        <v>50032683</v>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>好运包张</t>
+          <t>陆建军</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:55:37</t>
+          <t>2026-09-04 12:23:53</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="I35" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J35" s="0" t="inlineStr">
@@ -2170,11 +2170,11 @@
     </row>
     <row r="36" spans="1:14">
       <c r="A36" s="0">
-        <v>49984055</v>
+        <v>50015883</v>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>点点星辰</t>
+          <t>A00金华义乌叉车出租电15268650979</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:49:33</t>
+          <t>2026-09-03 23:18:02</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="I36" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J36" s="0" t="inlineStr">
@@ -2230,11 +2230,11 @@
     </row>
     <row r="37" spans="1:14">
       <c r="A37" s="0">
-        <v>49983134</v>
+        <v>50015882</v>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>Zhangrruzhen张如真</t>
+          <t>建程仓储中心 张川</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -2259,7 +2259,7 @@
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:25:21</t>
+          <t>2026-09-03 23:18:02</t>
         </is>
       </c>
       <c r="H37" s="0" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="I37" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J37" s="0" t="inlineStr">
@@ -2290,11 +2290,11 @@
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="0">
-        <v>49971209</v>
+        <v>50015784</v>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>顺丰顺水</t>
+          <t>天空</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:29:41</t>
+          <t>2026-09-03 23:10:41</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
@@ -2350,11 +2350,11 @@
     </row>
     <row r="39" spans="1:14">
       <c r="A39" s="0">
-        <v>49970732</v>
+        <v>50015778</v>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>小龙女</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:13:53</t>
+          <t>2026-09-03 23:10:21</t>
         </is>
       </c>
       <c r="H39" s="0" t="inlineStr">
@@ -2410,11 +2410,11 @@
     </row>
     <row r="40" spans="1:14">
       <c r="A40" s="0">
-        <v>49970712</v>
+        <v>50015776</v>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>月色琴弦</t>
+          <t>桥梁</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:13:07</t>
+          <t>2026-09-03 23:10:15</t>
         </is>
       </c>
       <c r="H40" s="0" t="inlineStr">
@@ -2470,11 +2470,11 @@
     </row>
     <row r="41" spans="1:14">
       <c r="A41" s="0">
-        <v>49970699</v>
+        <v>50015775</v>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>铜铃</t>
+          <t>彩云之南</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:49</t>
+          <t>2026-09-03 23:10:13</t>
         </is>
       </c>
       <c r="H41" s="0" t="inlineStr">
@@ -2530,11 +2530,11 @@
     </row>
     <row r="42" spans="1:14">
       <c r="A42" s="0">
-        <v>49970698</v>
+        <v>50015774</v>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>东风吹</t>
+          <t>楊精蓄銳༒</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:47</t>
+          <t>2026-09-03 23:10:11</t>
         </is>
       </c>
       <c r="H42" s="0" t="inlineStr">
@@ -2590,11 +2590,11 @@
     </row>
     <row r="43" spans="1:14">
       <c r="A43" s="0">
-        <v>49970683</v>
+        <v>50015772</v>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>杨永强</t>
+          <t>不倒翁</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:17</t>
+          <t>2026-09-03 23:10:07</t>
         </is>
       </c>
       <c r="H43" s="0" t="inlineStr">
@@ -2650,11 +2650,11 @@
     </row>
     <row r="44" spans="1:14">
       <c r="A44" s="0">
-        <v>49970662</v>
+        <v>50015770</v>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>盈丰</t>
+          <t>一江春水</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:33</t>
+          <t>2026-09-03 23:10:05</t>
         </is>
       </c>
       <c r="H44" s="0" t="inlineStr">
@@ -2710,11 +2710,11 @@
     </row>
     <row r="45" spans="1:14">
       <c r="A45" s="0">
-        <v>49970652</v>
+        <v>50015767</v>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>YAN</t>
+          <t>微笑</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:15</t>
+          <t>2026-09-03 23:10:03</t>
         </is>
       </c>
       <c r="H45" s="0" t="inlineStr">
@@ -2770,11 +2770,11 @@
     </row>
     <row r="46" spans="1:14">
       <c r="A46" s="0">
-        <v>49970649</v>
+        <v>50015763</v>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>彩虹（宋荷娣）</t>
+          <t>北斗星</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:11</t>
+          <t>2026-09-03 23:09:39</t>
         </is>
       </c>
       <c r="H46" s="0" t="inlineStr">
@@ -2830,11 +2830,11 @@
     </row>
     <row r="47" spans="1:14">
       <c r="A47" s="0">
-        <v>49970648</v>
+        <v>49989442</v>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>天知心</t>
+          <t>冬梅花儿开王丽君</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:08</t>
+          <t>2026-09-03 12:23:43</t>
         </is>
       </c>
       <c r="H47" s="0" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="I47" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J47" s="0" t="inlineStr">
@@ -2890,11 +2890,11 @@
     </row>
     <row r="48" spans="1:14">
       <c r="A48" s="0">
-        <v>49970643</v>
+        <v>49989431</v>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>好运来</t>
+          <t>风声</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:10:55</t>
+          <t>2026-09-03 12:23:25</t>
         </is>
       </c>
       <c r="H48" s="0" t="inlineStr">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="I48" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J48" s="0" t="inlineStr">
@@ -2950,11 +2950,11 @@
     </row>
     <row r="49" spans="1:14">
       <c r="A49" s="0">
-        <v>49937566</v>
+        <v>49989419</v>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>简单sincerity</t>
+          <t>胡宾</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 10:10:33</t>
+          <t>2026-09-03 12:23:13</t>
         </is>
       </c>
       <c r="H49" s="0" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="I49" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J49" s="0" t="inlineStr">
@@ -3010,11 +3010,11 @@
     </row>
     <row r="50" spans="1:14">
       <c r="A50" s="0">
-        <v>49937187</v>
+        <v>49989410</v>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>莲子</t>
+          <t>永远</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:58:56</t>
+          <t>2026-09-03 12:23:03</t>
         </is>
       </c>
       <c r="H50" s="0" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="I50" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J50" s="0" t="inlineStr">
@@ -3070,11 +3070,11 @@
     </row>
     <row r="51" spans="1:14">
       <c r="A51" s="0">
-        <v>49937101</v>
+        <v>49984259</v>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>蓉儿</t>
+          <t>好运包张</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:56:16</t>
+          <t>2026-09-03 09:55:37</t>
         </is>
       </c>
       <c r="H51" s="0" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="I51" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J51" s="0" t="inlineStr">
@@ -3130,11 +3130,11 @@
     </row>
     <row r="52" spans="1:14">
       <c r="A52" s="0">
-        <v>49937098</v>
+        <v>49984055</v>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>瀚林2368</t>
+          <t>点点星辰</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:56:15</t>
+          <t>2026-09-03 09:49:33</t>
         </is>
       </c>
       <c r="H52" s="0" t="inlineStr">
@@ -3190,11 +3190,11 @@
     </row>
     <row r="53" spans="1:14">
       <c r="A53" s="0">
-        <v>49937081</v>
+        <v>49983134</v>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>🔱 花中之美</t>
+          <t>Zhangrruzhen张如真</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:47</t>
+          <t>2026-09-03 09:25:21</t>
         </is>
       </c>
       <c r="H53" s="0" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="I53" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J53" s="0" t="inlineStr">
@@ -3250,11 +3250,11 @@
     </row>
     <row r="54" spans="1:14">
       <c r="A54" s="0">
-        <v>49937066</v>
+        <v>49971209</v>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>雨情</t>
+          <t>顺丰顺水</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:27</t>
+          <t>2026-09-02 23:29:41</t>
         </is>
       </c>
       <c r="H54" s="0" t="inlineStr">
@@ -3310,11 +3310,11 @@
     </row>
     <row r="55" spans="1:14">
       <c r="A55" s="0">
-        <v>49937061</v>
+        <v>49970732</v>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>Sunny 🎈瑶</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:23</t>
+          <t>2026-09-02 23:13:53</t>
         </is>
       </c>
       <c r="H55" s="0" t="inlineStr">
@@ -3370,11 +3370,11 @@
     </row>
     <row r="56" spans="1:14">
       <c r="A56" s="0">
-        <v>49887876</v>
+        <v>49970712</v>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>鱼靖儿</t>
+          <t>月色琴弦</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -3399,7 +3399,7 @@
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:23:11</t>
+          <t>2026-09-02 23:13:07</t>
         </is>
       </c>
       <c r="H56" s="0" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="I56" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J56" s="0" t="inlineStr">
@@ -3430,11 +3430,11 @@
     </row>
     <row r="57" spans="1:14">
       <c r="A57" s="0">
-        <v>49887478</v>
+        <v>49970699</v>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>风调雨顺</t>
+          <t>铜铃</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -3459,7 +3459,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:10:17</t>
+          <t>2026-09-02 23:12:49</t>
         </is>
       </c>
       <c r="H57" s="0" t="inlineStr">
@@ -3490,11 +3490,11 @@
     </row>
     <row r="58" spans="1:14">
       <c r="A58" s="0">
-        <v>49887447</v>
+        <v>49970698</v>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>中国艺人</t>
+          <t>东风吹</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:44</t>
+          <t>2026-09-02 23:12:47</t>
         </is>
       </c>
       <c r="H58" s="0" t="inlineStr">
@@ -3550,11 +3550,11 @@
     </row>
     <row r="59" spans="1:14">
       <c r="A59" s="0">
-        <v>49887439</v>
+        <v>49970683</v>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>黄晓玲</t>
+          <t>杨永强</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:17</t>
+          <t>2026-09-02 23:12:17</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
@@ -3610,11 +3610,11 @@
     </row>
     <row r="60" spans="1:14">
       <c r="A60" s="0">
-        <v>49887437</v>
+        <v>49970662</v>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>随缘</t>
+          <t>盈丰</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:07</t>
+          <t>2026-09-02 23:11:33</t>
         </is>
       </c>
       <c r="H60" s="0" t="inlineStr">
@@ -3670,11 +3670,11 @@
     </row>
     <row r="61" spans="1:14">
       <c r="A61" s="0">
-        <v>49887416</v>
+        <v>49970652</v>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>刘秋红</t>
+          <t>YAN</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:31</t>
+          <t>2026-09-02 23:11:15</t>
         </is>
       </c>
       <c r="H61" s="0" t="inlineStr">
@@ -3730,11 +3730,11 @@
     </row>
     <row r="62" spans="1:14">
       <c r="A62" s="0">
-        <v>49887403</v>
+        <v>49970649</v>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>Mr.</t>
+          <t>彩虹（宋荷娣）</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:05</t>
+          <t>2026-09-02 23:11:11</t>
         </is>
       </c>
       <c r="H62" s="0" t="inlineStr">
@@ -3790,11 +3790,11 @@
     </row>
     <row r="63" spans="1:14">
       <c r="A63" s="0">
-        <v>49887401</v>
+        <v>49970648</v>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>万事如意</t>
+          <t>天知心</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:03</t>
+          <t>2026-09-02 23:11:08</t>
         </is>
       </c>
       <c r="H63" s="0" t="inlineStr">
@@ -3850,11 +3850,11 @@
     </row>
     <row r="64" spans="1:14">
       <c r="A64" s="0">
-        <v>49887400</v>
+        <v>49970643</v>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>💋诺墨</t>
+          <t>好运来</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:01</t>
+          <t>2026-09-02 23:10:55</t>
         </is>
       </c>
       <c r="H64" s="0" t="inlineStr">
@@ -3910,11 +3910,11 @@
     </row>
     <row r="65" spans="1:14">
       <c r="A65" s="0">
-        <v>49887399</v>
+        <v>49937566</v>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>听风</t>
+          <t>简单sincerity</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:06:59</t>
+          <t>2026-09-02 10:10:33</t>
         </is>
       </c>
       <c r="H65" s="0" t="inlineStr">
@@ -3970,11 +3970,11 @@
     </row>
     <row r="66" spans="1:14">
       <c r="A66" s="0">
-        <v>49845584</v>
+        <v>49937187</v>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>彭汉平13024282926</t>
+          <t>莲子</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:18:55</t>
+          <t>2026-09-02 09:58:56</t>
         </is>
       </c>
       <c r="H66" s="0" t="inlineStr">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="I66" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J66" s="0" t="inlineStr">
@@ -4030,11 +4030,11 @@
     </row>
     <row r="67" spans="1:14">
       <c r="A67" s="0">
-        <v>49845487</v>
+        <v>49937101</v>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>Z国华</t>
+          <t>蓉儿</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:15:49</t>
+          <t>2026-09-02 09:56:16</t>
         </is>
       </c>
       <c r="H67" s="0" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="I67" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J67" s="0" t="inlineStr">
@@ -4090,11 +4090,11 @@
     </row>
     <row r="68" spans="1:14">
       <c r="A68" s="0">
-        <v>49845407</v>
+        <v>49937098</v>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>月亮🌛</t>
+          <t>瀚林2368</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:12:33</t>
+          <t>2026-09-02 09:56:15</t>
         </is>
       </c>
       <c r="H68" s="0" t="inlineStr">
@@ -4150,11 +4150,11 @@
     </row>
     <row r="69" spans="1:14">
       <c r="A69" s="0">
-        <v>49845398</v>
+        <v>49937081</v>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>老树</t>
+          <t>🔱 花中之美</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:12:03</t>
+          <t>2026-09-02 09:55:47</t>
         </is>
       </c>
       <c r="H69" s="0" t="inlineStr">
@@ -4210,11 +4210,11 @@
     </row>
     <row r="70" spans="1:14">
       <c r="A70" s="0">
-        <v>49845391</v>
+        <v>49937066</v>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>八哥</t>
+          <t>雨情</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:45</t>
+          <t>2026-09-02 09:55:27</t>
         </is>
       </c>
       <c r="H70" s="0" t="inlineStr">
@@ -4270,11 +4270,11 @@
     </row>
     <row r="71" spans="1:14">
       <c r="A71" s="0">
-        <v>49845380</v>
+        <v>49937061</v>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>铲车主出租15352562068</t>
+          <t>Sunny 🎈瑶</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -4299,7 +4299,7 @@
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:29</t>
+          <t>2026-09-02 09:55:23</t>
         </is>
       </c>
       <c r="H71" s="0" t="inlineStr">
@@ -4330,11 +4330,11 @@
     </row>
     <row r="72" spans="1:14">
       <c r="A72" s="0">
-        <v>49845376</v>
+        <v>49887876</v>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>刘萍</t>
+          <t>鱼靖儿</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -4359,7 +4359,7 @@
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:15</t>
+          <t>2026-08-31 23:23:11</t>
         </is>
       </c>
       <c r="H72" s="0" t="inlineStr">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="I72" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J72" s="0" t="inlineStr">
@@ -4390,11 +4390,11 @@
     </row>
     <row r="73" spans="1:14">
       <c r="A73" s="0">
-        <v>49845374</v>
+        <v>49887478</v>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>空谷幽兰</t>
+          <t>风调雨顺</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:07</t>
+          <t>2026-08-31 23:10:17</t>
         </is>
       </c>
       <c r="H73" s="0" t="inlineStr">
@@ -4450,11 +4450,11 @@
     </row>
     <row r="74" spans="1:14">
       <c r="A74" s="0">
-        <v>49845373</v>
+        <v>49887447</v>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>泽浩羊</t>
+          <t>中国艺人</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:05</t>
+          <t>2026-08-31 23:08:44</t>
         </is>
       </c>
       <c r="H74" s="0" t="inlineStr">
@@ -4510,11 +4510,11 @@
     </row>
     <row r="75" spans="1:14">
       <c r="A75" s="0">
-        <v>49845367</v>
+        <v>49887439</v>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>峰回路转</t>
+          <t>黄晓玲</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -4539,7 +4539,7 @@
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:55</t>
+          <t>2026-08-31 23:08:17</t>
         </is>
       </c>
       <c r="H75" s="0" t="inlineStr">
@@ -4570,11 +4570,11 @@
     </row>
     <row r="76" spans="1:14">
       <c r="A76" s="0">
-        <v>49845366</v>
+        <v>49887437</v>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>超儿</t>
+          <t>随缘</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -4599,7 +4599,7 @@
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:51</t>
+          <t>2026-08-31 23:08:07</t>
         </is>
       </c>
       <c r="H76" s="0" t="inlineStr">
@@ -4630,11 +4630,11 @@
     </row>
     <row r="77" spans="1:14">
       <c r="A77" s="0">
-        <v>49845365</v>
+        <v>49887416</v>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>传</t>
+          <t>刘秋红</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -4659,7 +4659,7 @@
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:49</t>
+          <t>2026-08-31 23:07:31</t>
         </is>
       </c>
       <c r="H77" s="0" t="inlineStr">
@@ -4690,11 +4690,11 @@
     </row>
     <row r="78" spans="1:14">
       <c r="A78" s="0">
-        <v>49845360</v>
+        <v>49887403</v>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>悟歌</t>
+          <t>Mr.</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -4719,7 +4719,7 @@
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:43</t>
+          <t>2026-08-31 23:07:05</t>
         </is>
       </c>
       <c r="H78" s="0" t="inlineStr">
@@ -4750,11 +4750,11 @@
     </row>
     <row r="79" spans="1:14">
       <c r="A79" s="0">
-        <v>49845342</v>
+        <v>49887401</v>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>丽丽</t>
+          <t>万事如意</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -4779,7 +4779,7 @@
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:15</t>
+          <t>2026-08-31 23:07:03</t>
         </is>
       </c>
       <c r="H79" s="0" t="inlineStr">
@@ -4810,11 +4810,11 @@
     </row>
     <row r="80" spans="1:14">
       <c r="A80" s="0">
-        <v>49826011</v>
+        <v>49887400</v>
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>王前卫</t>
+          <t>💋诺墨</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:57:27</t>
+          <t>2026-08-31 23:07:01</t>
         </is>
       </c>
       <c r="H80" s="0" t="inlineStr">
@@ -4870,11 +4870,11 @@
     </row>
     <row r="81" spans="1:14">
       <c r="A81" s="0">
-        <v>49825720</v>
+        <v>49887399</v>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>老A</t>
+          <t>听风</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:46:02</t>
+          <t>2026-08-31 23:06:59</t>
         </is>
       </c>
       <c r="H81" s="0" t="inlineStr">
@@ -4930,11 +4930,11 @@
     </row>
     <row r="82" spans="1:14">
       <c r="A82" s="0">
-        <v>49825676</v>
+        <v>49845584</v>
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>蓝天</t>
+          <t>彭汉平13024282926</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:44:05</t>
+          <t>2026-08-30 23:18:55</t>
         </is>
       </c>
       <c r="H82" s="0" t="inlineStr">
@@ -4990,11 +4990,11 @@
     </row>
     <row r="83" spans="1:14">
       <c r="A83" s="0">
-        <v>49825650</v>
+        <v>49845487</v>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>爱芳</t>
+          <t>Z国华</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -5019,7 +5019,7 @@
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:43:11</t>
+          <t>2026-08-30 23:15:49</t>
         </is>
       </c>
       <c r="H83" s="0" t="inlineStr">
@@ -5029,7 +5029,7 @@
       </c>
       <c r="I83" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J83" s="0" t="inlineStr">
@@ -5050,11 +5050,11 @@
     </row>
     <row r="84" spans="1:14">
       <c r="A84" s="0">
-        <v>49825642</v>
+        <v>49845407</v>
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>银杏树</t>
+          <t>月亮🌛</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -5079,7 +5079,7 @@
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:55</t>
+          <t>2026-08-30 23:12:33</t>
         </is>
       </c>
       <c r="H84" s="0" t="inlineStr">
@@ -5110,11 +5110,11 @@
     </row>
     <row r="85" spans="1:14">
       <c r="A85" s="0">
-        <v>49825640</v>
+        <v>49845398</v>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>遵命有福（杨凤）</t>
+          <t>老树</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:49</t>
+          <t>2026-08-30 23:12:03</t>
         </is>
       </c>
       <c r="H85" s="0" t="inlineStr">
@@ -5170,11 +5170,11 @@
     </row>
     <row r="86" spans="1:14">
       <c r="A86" s="0">
-        <v>49825639</v>
+        <v>49845391</v>
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>申华</t>
+          <t>八哥</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -5199,7 +5199,7 @@
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:49</t>
+          <t>2026-08-30 23:11:45</t>
         </is>
       </c>
       <c r="H86" s="0" t="inlineStr">
@@ -5230,11 +5230,11 @@
     </row>
     <row r="87" spans="1:14">
       <c r="A87" s="0">
-        <v>49825637</v>
+        <v>49845380</v>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>陈月焓</t>
+          <t>铲车主出租15352562068</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:47</t>
+          <t>2026-08-30 23:11:29</t>
         </is>
       </c>
       <c r="H87" s="0" t="inlineStr">
@@ -5290,11 +5290,11 @@
     </row>
     <row r="88" spans="1:14">
       <c r="A88" s="0">
-        <v>49825635</v>
+        <v>49845376</v>
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>小镇生活&amp;&amp;杜震</t>
+          <t>刘萍</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -5319,7 +5319,7 @@
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:43</t>
+          <t>2026-08-30 23:11:15</t>
         </is>
       </c>
       <c r="H88" s="0" t="inlineStr">
@@ -5350,11 +5350,11 @@
     </row>
     <row r="89" spans="1:14">
       <c r="A89" s="0">
-        <v>49825628</v>
+        <v>49845374</v>
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>Taᴗaoᥫᩣ</t>
+          <t>空谷幽兰</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:35</t>
+          <t>2026-08-30 23:11:07</t>
         </is>
       </c>
       <c r="H89" s="0" t="inlineStr">
@@ -5410,11 +5410,11 @@
     </row>
     <row r="90" spans="1:14">
       <c r="A90" s="0">
-        <v>49782066</v>
+        <v>49845373</v>
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>前程似锦</t>
+          <t>泽浩羊</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 09:07:29</t>
+          <t>2026-08-30 23:11:05</t>
         </is>
       </c>
       <c r="H90" s="0" t="inlineStr">
@@ -5449,7 +5449,7 @@
       </c>
       <c r="I90" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J90" s="0" t="inlineStr">
@@ -5470,11 +5470,11 @@
     </row>
     <row r="91" spans="1:14">
       <c r="A91" s="0">
-        <v>49771027</v>
+        <v>49845367</v>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>非比</t>
+          <t>峰回路转</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -5499,7 +5499,7 @@
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 23:30:09</t>
+          <t>2026-08-30 23:10:55</t>
         </is>
       </c>
       <c r="H91" s="0" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="I91" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J91" s="0" t="inlineStr">
@@ -5530,11 +5530,11 @@
     </row>
     <row r="92" spans="1:14">
       <c r="A92" s="0">
-        <v>49673360</v>
+        <v>49845366</v>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t>德行天下</t>
+          <t>超儿</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="G92" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:19:03</t>
+          <t>2026-08-30 23:10:51</t>
         </is>
       </c>
       <c r="H92" s="0" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="I92" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J92" s="0" t="inlineStr">
@@ -5590,11 +5590,11 @@
     </row>
     <row r="93" spans="1:14">
       <c r="A93" s="0">
-        <v>49673352</v>
+        <v>49845365</v>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t>余盛将至2026</t>
+          <t>传</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -5619,7 +5619,7 @@
       </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:49</t>
+          <t>2026-08-30 23:10:49</t>
         </is>
       </c>
       <c r="H93" s="0" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="I93" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J93" s="0" t="inlineStr">
@@ -5650,11 +5650,11 @@
     </row>
     <row r="94" spans="1:14">
       <c r="A94" s="0">
-        <v>49673350</v>
+        <v>49845360</v>
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t>山居客</t>
+          <t>悟歌</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
@@ -5679,7 +5679,7 @@
       </c>
       <c r="G94" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:47</t>
+          <t>2026-08-30 23:10:43</t>
         </is>
       </c>
       <c r="H94" s="0" t="inlineStr">
@@ -5689,7 +5689,7 @@
       </c>
       <c r="I94" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J94" s="0" t="inlineStr">
@@ -5710,11 +5710,11 @@
     </row>
     <row r="95" spans="1:14">
       <c r="A95" s="0">
-        <v>49673349</v>
+        <v>49845342</v>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>白云</t>
+          <t>丽丽</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="G95" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:45</t>
+          <t>2026-08-30 23:10:15</t>
         </is>
       </c>
       <c r="H95" s="0" t="inlineStr">
@@ -5749,7 +5749,7 @@
       </c>
       <c r="I95" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J95" s="0" t="inlineStr">
@@ -5770,11 +5770,11 @@
     </row>
     <row r="96" spans="1:14">
       <c r="A96" s="0">
-        <v>49646935</v>
+        <v>49826011</v>
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t>马跃荣</t>
+          <t>王前卫</t>
         </is>
       </c>
       <c r="C96" s="0" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="G96" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:59</t>
+          <t>2026-08-30 12:57:27</t>
         </is>
       </c>
       <c r="H96" s="0" t="inlineStr">
@@ -5809,7 +5809,7 @@
       </c>
       <c r="I96" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J96" s="0" t="inlineStr">
@@ -5830,11 +5830,11 @@
     </row>
     <row r="97" spans="1:14">
       <c r="A97" s="0">
-        <v>49646933</v>
+        <v>49825720</v>
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>@吴</t>
+          <t>老A</t>
         </is>
       </c>
       <c r="C97" s="0" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="G97" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:56</t>
+          <t>2026-08-30 12:46:02</t>
         </is>
       </c>
       <c r="H97" s="0" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="I97" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J97" s="0" t="inlineStr">
@@ -5890,11 +5890,11 @@
     </row>
     <row r="98" spans="1:14">
       <c r="A98" s="0">
-        <v>49646901</v>
+        <v>49825676</v>
       </c>
       <c r="B98" s="0" t="inlineStr">
         <is>
-          <t>龙安：富华／</t>
+          <t>蓝天</t>
         </is>
       </c>
       <c r="C98" s="0" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="G98" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:14:28</t>
+          <t>2026-08-30 12:44:05</t>
         </is>
       </c>
       <c r="H98" s="0" t="inlineStr">
@@ -5929,7 +5929,7 @@
       </c>
       <c r="I98" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J98" s="0" t="inlineStr">
@@ -5950,11 +5950,11 @@
     </row>
     <row r="99" spans="1:14">
       <c r="A99" s="0">
-        <v>49646876</v>
+        <v>49825650</v>
       </c>
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t>冬日暖阳🌻</t>
+          <t>爱芳</t>
         </is>
       </c>
       <c r="C99" s="0" t="inlineStr">
@@ -5979,7 +5979,7 @@
       </c>
       <c r="G99" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:37</t>
+          <t>2026-08-30 12:43:11</t>
         </is>
       </c>
       <c r="H99" s="0" t="inlineStr">
@@ -5989,7 +5989,7 @@
       </c>
       <c r="I99" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J99" s="0" t="inlineStr">
@@ -6010,11 +6010,11 @@
     </row>
     <row r="100" spans="1:14">
       <c r="A100" s="0">
-        <v>49646867</v>
+        <v>49825642</v>
       </c>
       <c r="B100" s="0" t="inlineStr">
         <is>
-          <t>寒雨</t>
+          <t>银杏树</t>
         </is>
       </c>
       <c r="C100" s="0" t="inlineStr">
@@ -6039,7 +6039,7 @@
       </c>
       <c r="G100" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:15</t>
+          <t>2026-08-30 12:42:55</t>
         </is>
       </c>
       <c r="H100" s="0" t="inlineStr">
@@ -6049,7 +6049,7 @@
       </c>
       <c r="I100" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J100" s="0" t="inlineStr">
@@ -6070,11 +6070,11 @@
     </row>
     <row r="101" spans="1:14">
       <c r="A101" s="0">
-        <v>49636232</v>
+        <v>49825640</v>
       </c>
       <c r="B101" s="0" t="inlineStr">
         <is>
-          <t>平安</t>
+          <t>遵命有福（杨凤）</t>
         </is>
       </c>
       <c r="C101" s="0" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="G101" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:20:15</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H101" s="0" t="inlineStr">
@@ -6109,7 +6109,7 @@
       </c>
       <c r="I101" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J101" s="0" t="inlineStr">
@@ -6130,11 +6130,11 @@
     </row>
     <row r="102" spans="1:14">
       <c r="A102" s="0">
-        <v>49636184</v>
+        <v>49825639</v>
       </c>
       <c r="B102" s="0" t="inlineStr">
         <is>
-          <t>古道西风</t>
+          <t>申华</t>
         </is>
       </c>
       <c r="C102" s="0" t="inlineStr">
@@ -6159,7 +6159,7 @@
       </c>
       <c r="G102" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:55</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H102" s="0" t="inlineStr">
@@ -6190,11 +6190,11 @@
     </row>
     <row r="103" spans="1:14">
       <c r="A103" s="0">
-        <v>49636170</v>
+        <v>49825637</v>
       </c>
       <c r="B103" s="0" t="inlineStr">
         <is>
-          <t>周海龙</t>
+          <t>陈月焓</t>
         </is>
       </c>
       <c r="C103" s="0" t="inlineStr">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="G103" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:33</t>
+          <t>2026-08-30 12:42:47</t>
         </is>
       </c>
       <c r="H103" s="0" t="inlineStr">
@@ -6250,11 +6250,11 @@
     </row>
     <row r="104" spans="1:14">
       <c r="A104" s="0">
-        <v>49636157</v>
+        <v>49825635</v>
       </c>
       <c r="B104" s="0" t="inlineStr">
         <is>
-          <t>锦妍</t>
+          <t>小镇生活&amp;&amp;杜震</t>
         </is>
       </c>
       <c r="C104" s="0" t="inlineStr">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="G104" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:07</t>
+          <t>2026-08-30 12:42:43</t>
         </is>
       </c>
       <c r="H104" s="0" t="inlineStr">
@@ -6310,11 +6310,11 @@
     </row>
     <row r="105" spans="1:14">
       <c r="A105" s="0">
-        <v>49593974</v>
+        <v>49825628</v>
       </c>
       <c r="B105" s="0" t="inlineStr">
         <is>
-          <t>兰兰</t>
+          <t>Taᴗaoᥫᩣ</t>
         </is>
       </c>
       <c r="C105" s="0" t="inlineStr">
@@ -6339,7 +6339,7 @@
       </c>
       <c r="G105" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:59:53</t>
+          <t>2026-08-30 12:42:35</t>
         </is>
       </c>
       <c r="H105" s="0" t="inlineStr">
@@ -6349,7 +6349,7 @@
       </c>
       <c r="I105" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J105" s="0" t="inlineStr">
@@ -6370,11 +6370,11 @@
     </row>
     <row r="106" spans="1:14">
       <c r="A106" s="0">
-        <v>49593671</v>
+        <v>49782066</v>
       </c>
       <c r="B106" s="0" t="inlineStr">
         <is>
-          <t>准备1号</t>
+          <t>前程似锦</t>
         </is>
       </c>
       <c r="C106" s="0" t="inlineStr">
@@ -6399,7 +6399,7 @@
       </c>
       <c r="G106" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:49:27</t>
+          <t>2026-08-29 09:07:29</t>
         </is>
       </c>
       <c r="H106" s="0" t="inlineStr">
@@ -6430,11 +6430,11 @@
     </row>
     <row r="107" spans="1:14">
       <c r="A107" s="0">
-        <v>49535916</v>
+        <v>49771027</v>
       </c>
       <c r="B107" s="0" t="inlineStr">
         <is>
-          <t>真诚</t>
+          <t>非比</t>
         </is>
       </c>
       <c r="C107" s="0" t="inlineStr">
@@ -6459,7 +6459,7 @@
       </c>
       <c r="G107" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:46:23</t>
+          <t>2026-08-28 23:30:09</t>
         </is>
       </c>
       <c r="H107" s="0" t="inlineStr">
@@ -6490,11 +6490,11 @@
     </row>
     <row r="108" spans="1:14">
       <c r="A108" s="0">
-        <v>49535653</v>
+        <v>49673360</v>
       </c>
       <c r="B108" s="0" t="inlineStr">
         <is>
-          <t>如意家电13368134456维修</t>
+          <t>德行天下</t>
         </is>
       </c>
       <c r="C108" s="0" t="inlineStr">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="G108" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:28:25</t>
+          <t>2026-08-26 12:19:03</t>
         </is>
       </c>
       <c r="H108" s="0" t="inlineStr">
@@ -6529,7 +6529,7 @@
       </c>
       <c r="I108" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J108" s="0" t="inlineStr">
@@ -6550,11 +6550,11 @@
     </row>
     <row r="109" spans="1:14">
       <c r="A109" s="0">
-        <v>49535650</v>
+        <v>49673352</v>
       </c>
       <c r="B109" s="0" t="inlineStr">
         <is>
-          <t>莺莺</t>
+          <t>余盛将至2026</t>
         </is>
       </c>
       <c r="C109" s="0" t="inlineStr">
@@ -6579,7 +6579,7 @@
       </c>
       <c r="G109" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:27:55</t>
+          <t>2026-08-26 12:18:49</t>
         </is>
       </c>
       <c r="H109" s="0" t="inlineStr">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="I109" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J109" s="0" t="inlineStr">
@@ -6605,21 +6605,16 @@
       <c r="L109" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N109" s="0" t="inlineStr">
-        <is>
-          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="110" spans="1:14">
       <c r="A110" s="0">
-        <v>49508265</v>
+        <v>49673350</v>
       </c>
       <c r="B110" s="0" t="inlineStr">
         <is>
-          <t>爱猫🐱 咪</t>
+          <t>山居客</t>
         </is>
       </c>
       <c r="C110" s="0" t="inlineStr">
@@ -6644,7 +6639,7 @@
       </c>
       <c r="G110" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 09:53:41</t>
+          <t>2026-08-26 12:18:47</t>
         </is>
       </c>
       <c r="H110" s="0" t="inlineStr">
@@ -6654,7 +6649,7 @@
       </c>
       <c r="I110" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J110" s="0" t="inlineStr">
@@ -6675,11 +6670,11 @@
     </row>
     <row r="111" spans="1:14">
       <c r="A111" s="0">
-        <v>49493414</v>
+        <v>49673349</v>
       </c>
       <c r="B111" s="0" t="inlineStr">
         <is>
-          <t>惠平</t>
+          <t>白云</t>
         </is>
       </c>
       <c r="C111" s="0" t="inlineStr">
@@ -6704,7 +6699,7 @@
       </c>
       <c r="G111" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:53:02</t>
+          <t>2026-08-26 12:18:45</t>
         </is>
       </c>
       <c r="H111" s="0" t="inlineStr">
@@ -6714,7 +6709,7 @@
       </c>
       <c r="I111" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J111" s="0" t="inlineStr">
@@ -6735,11 +6730,11 @@
     </row>
     <row r="112" spans="1:14">
       <c r="A112" s="0">
-        <v>49493126</v>
+        <v>49646935</v>
       </c>
       <c r="B112" s="0" t="inlineStr">
         <is>
-          <t>刘盼昭</t>
+          <t>马跃荣</t>
         </is>
       </c>
       <c r="C112" s="0" t="inlineStr">
@@ -6764,7 +6759,7 @@
       </c>
       <c r="G112" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:44:53</t>
+          <t>2026-08-25 18:15:59</t>
         </is>
       </c>
       <c r="H112" s="0" t="inlineStr">
@@ -6774,7 +6769,7 @@
       </c>
       <c r="I112" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J112" s="0" t="inlineStr">
@@ -6795,11 +6790,11 @@
     </row>
     <row r="113" spans="1:14">
       <c r="A113" s="0">
-        <v>49492499</v>
+        <v>49646933</v>
       </c>
       <c r="B113" s="0" t="inlineStr">
         <is>
-          <t>红霞</t>
+          <t>@吴</t>
         </is>
       </c>
       <c r="C113" s="0" t="inlineStr">
@@ -6824,7 +6819,7 @@
       </c>
       <c r="G113" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:29:43</t>
+          <t>2026-08-25 18:15:56</t>
         </is>
       </c>
       <c r="H113" s="0" t="inlineStr">
@@ -6834,7 +6829,7 @@
       </c>
       <c r="I113" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J113" s="0" t="inlineStr">
@@ -6855,11 +6850,11 @@
     </row>
     <row r="114" spans="1:14">
       <c r="A114" s="0">
-        <v>49455301</v>
+        <v>49646901</v>
       </c>
       <c r="B114" s="0" t="inlineStr">
         <is>
-          <t>周开平</t>
+          <t>龙安：富华／</t>
         </is>
       </c>
       <c r="C114" s="0" t="inlineStr">
@@ -6884,7 +6879,7 @@
       </c>
       <c r="G114" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 22:46:59</t>
+          <t>2026-08-25 18:14:28</t>
         </is>
       </c>
       <c r="H114" s="0" t="inlineStr">
@@ -6894,7 +6889,7 @@
       </c>
       <c r="I114" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J114" s="0" t="inlineStr">
@@ -6915,11 +6910,11 @@
     </row>
     <row r="115" spans="1:14">
       <c r="A115" s="0">
-        <v>49432023</v>
+        <v>49646876</v>
       </c>
       <c r="B115" s="0" t="inlineStr">
         <is>
-          <t>花生米</t>
+          <t>冬日暖阳🌻</t>
         </is>
       </c>
       <c r="C115" s="0" t="inlineStr">
@@ -6944,7 +6939,7 @@
       </c>
       <c r="G115" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 11:55:45</t>
+          <t>2026-08-25 18:13:37</t>
         </is>
       </c>
       <c r="H115" s="0" t="inlineStr">
@@ -6954,7 +6949,7 @@
       </c>
       <c r="I115" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J115" s="0" t="inlineStr">
@@ -6975,11 +6970,11 @@
     </row>
     <row r="116" spans="1:14">
       <c r="A116" s="0">
-        <v>49415939</v>
+        <v>49646867</v>
       </c>
       <c r="B116" s="0" t="inlineStr">
         <is>
-          <t>杨梅芳</t>
+          <t>寒雨</t>
         </is>
       </c>
       <c r="C116" s="0" t="inlineStr">
@@ -7004,7 +6999,7 @@
       </c>
       <c r="G116" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:58</t>
+          <t>2026-08-25 18:13:15</t>
         </is>
       </c>
       <c r="H116" s="0" t="inlineStr">
@@ -7014,17 +7009,17 @@
       </c>
       <c r="I116" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J116" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K116" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L116" s="0" t="inlineStr">
@@ -7035,11 +7030,11 @@
     </row>
     <row r="117" spans="1:14">
       <c r="A117" s="0">
-        <v>49415918</v>
+        <v>49636232</v>
       </c>
       <c r="B117" s="0" t="inlineStr">
         <is>
-          <t>心语无言</t>
+          <t>平安</t>
         </is>
       </c>
       <c r="C117" s="0" t="inlineStr">
@@ -7064,7 +7059,7 @@
       </c>
       <c r="G117" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:24</t>
+          <t>2026-08-25 13:20:15</t>
         </is>
       </c>
       <c r="H117" s="0" t="inlineStr">
@@ -7074,17 +7069,17 @@
       </c>
       <c r="I117" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J117" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K117" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L117" s="0" t="inlineStr">
@@ -7095,11 +7090,11 @@
     </row>
     <row r="118" spans="1:14">
       <c r="A118" s="0">
-        <v>49415913</v>
+        <v>49636184</v>
       </c>
       <c r="B118" s="0" t="inlineStr">
         <is>
-          <t>安好</t>
+          <t>古道西风</t>
         </is>
       </c>
       <c r="C118" s="0" t="inlineStr">
@@ -7124,7 +7119,7 @@
       </c>
       <c r="G118" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:18</t>
+          <t>2026-08-25 13:18:55</t>
         </is>
       </c>
       <c r="H118" s="0" t="inlineStr">
@@ -7139,12 +7134,12 @@
       </c>
       <c r="J118" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K118" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L118" s="0" t="inlineStr">
@@ -7155,11 +7150,11 @@
     </row>
     <row r="119" spans="1:14">
       <c r="A119" s="0">
-        <v>49415890</v>
+        <v>49636170</v>
       </c>
       <c r="B119" s="0" t="inlineStr">
         <is>
-          <t>雨夜聆风</t>
+          <t>周海龙</t>
         </is>
       </c>
       <c r="C119" s="0" t="inlineStr">
@@ -7184,7 +7179,7 @@
       </c>
       <c r="G119" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:56</t>
+          <t>2026-08-25 13:18:33</t>
         </is>
       </c>
       <c r="H119" s="0" t="inlineStr">
@@ -7199,32 +7194,27 @@
       </c>
       <c r="J119" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K119" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L119" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N119" s="0" t="inlineStr">
-        <is>
-          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="120" spans="1:14">
       <c r="A120" s="0">
-        <v>49415874</v>
+        <v>49636157</v>
       </c>
       <c r="B120" s="0" t="inlineStr">
         <is>
-          <t>飘</t>
+          <t>锦妍</t>
         </is>
       </c>
       <c r="C120" s="0" t="inlineStr">
@@ -7249,7 +7239,7 @@
       </c>
       <c r="G120" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:40</t>
+          <t>2026-08-25 13:18:07</t>
         </is>
       </c>
       <c r="H120" s="0" t="inlineStr">
@@ -7264,12 +7254,12 @@
       </c>
       <c r="J120" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K120" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L120" s="0" t="inlineStr">
@@ -7280,11 +7270,11 @@
     </row>
     <row r="121" spans="1:14">
       <c r="A121" s="0">
-        <v>49415871</v>
+        <v>49593974</v>
       </c>
       <c r="B121" s="0" t="inlineStr">
         <is>
-          <t>庆</t>
+          <t>兰兰</t>
         </is>
       </c>
       <c r="C121" s="0" t="inlineStr">
@@ -7309,7 +7299,7 @@
       </c>
       <c r="G121" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:36</t>
+          <t>2026-08-24 12:59:53</t>
         </is>
       </c>
       <c r="H121" s="0" t="inlineStr">
@@ -7319,17 +7309,17 @@
       </c>
       <c r="I121" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J121" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K121" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L121" s="0" t="inlineStr">
@@ -7340,59 +7330,1029 @@
     </row>
     <row r="122" spans="1:14">
       <c r="A122" s="0">
+        <v>49593671</v>
+      </c>
+      <c r="B122" s="0" t="inlineStr">
+        <is>
+          <t>准备1号</t>
+        </is>
+      </c>
+      <c r="C122" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D122" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E122" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F122" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G122" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-24 12:49:27</t>
+        </is>
+      </c>
+      <c r="H122" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I122" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J122" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K122" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L122" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" spans="1:14">
+      <c r="A123" s="0">
+        <v>49535916</v>
+      </c>
+      <c r="B123" s="0" t="inlineStr">
+        <is>
+          <t>真诚</t>
+        </is>
+      </c>
+      <c r="C123" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D123" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E123" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F123" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G123" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 23:46:23</t>
+        </is>
+      </c>
+      <c r="H123" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I123" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J123" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K123" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L123" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" spans="1:14">
+      <c r="A124" s="0">
+        <v>49535653</v>
+      </c>
+      <c r="B124" s="0" t="inlineStr">
+        <is>
+          <t>如意家电13368134456维修</t>
+        </is>
+      </c>
+      <c r="C124" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D124" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E124" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F124" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G124" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 23:28:25</t>
+        </is>
+      </c>
+      <c r="H124" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I124" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J124" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K124" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L124" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" spans="1:14">
+      <c r="A125" s="0">
+        <v>49535650</v>
+      </c>
+      <c r="B125" s="0" t="inlineStr">
+        <is>
+          <t>莺莺</t>
+        </is>
+      </c>
+      <c r="C125" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D125" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E125" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F125" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G125" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 23:27:55</t>
+        </is>
+      </c>
+      <c r="H125" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I125" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J125" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K125" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L125" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="N125" s="0" t="inlineStr">
+        <is>
+          <t>黄浦</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" spans="1:14">
+      <c r="A126" s="0">
+        <v>49508265</v>
+      </c>
+      <c r="B126" s="0" t="inlineStr">
+        <is>
+          <t>爱猫🐱 咪</t>
+        </is>
+      </c>
+      <c r="C126" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D126" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E126" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F126" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G126" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-22 09:53:41</t>
+        </is>
+      </c>
+      <c r="H126" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I126" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J126" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K126" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L126" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" spans="1:14">
+      <c r="A127" s="0">
+        <v>49493414</v>
+      </c>
+      <c r="B127" s="0" t="inlineStr">
+        <is>
+          <t>惠平</t>
+        </is>
+      </c>
+      <c r="C127" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D127" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E127" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F127" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G127" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-21 22:53:02</t>
+        </is>
+      </c>
+      <c r="H127" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I127" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J127" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K127" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L127" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" spans="1:14">
+      <c r="A128" s="0">
+        <v>49493126</v>
+      </c>
+      <c r="B128" s="0" t="inlineStr">
+        <is>
+          <t>刘盼昭</t>
+        </is>
+      </c>
+      <c r="C128" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D128" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E128" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F128" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G128" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-21 22:44:53</t>
+        </is>
+      </c>
+      <c r="H128" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I128" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J128" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K128" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L128" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" spans="1:14">
+      <c r="A129" s="0">
+        <v>49492499</v>
+      </c>
+      <c r="B129" s="0" t="inlineStr">
+        <is>
+          <t>红霞</t>
+        </is>
+      </c>
+      <c r="C129" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D129" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E129" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F129" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G129" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-21 22:29:43</t>
+        </is>
+      </c>
+      <c r="H129" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I129" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J129" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K129" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L129" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" spans="1:14">
+      <c r="A130" s="0">
+        <v>49455301</v>
+      </c>
+      <c r="B130" s="0" t="inlineStr">
+        <is>
+          <t>周开平</t>
+        </is>
+      </c>
+      <c r="C130" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D130" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E130" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F130" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G130" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-20 22:46:59</t>
+        </is>
+      </c>
+      <c r="H130" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I130" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J130" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K130" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L130" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" spans="1:14">
+      <c r="A131" s="0">
+        <v>49432023</v>
+      </c>
+      <c r="B131" s="0" t="inlineStr">
+        <is>
+          <t>花生米</t>
+        </is>
+      </c>
+      <c r="C131" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D131" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E131" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F131" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G131" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-20 11:55:45</t>
+        </is>
+      </c>
+      <c r="H131" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I131" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-视频号01</t>
+        </is>
+      </c>
+      <c r="J131" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-获客助手专用</t>
+        </is>
+      </c>
+      <c r="K131" s="0" t="inlineStr">
+        <is>
+          <t>获客助手加好友</t>
+        </is>
+      </c>
+      <c r="L131" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" spans="1:14">
+      <c r="A132" s="0">
+        <v>49415939</v>
+      </c>
+      <c r="B132" s="0" t="inlineStr">
+        <is>
+          <t>杨梅芳</t>
+        </is>
+      </c>
+      <c r="C132" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D132" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E132" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F132" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G132" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:58</t>
+        </is>
+      </c>
+      <c r="H132" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I132" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J132" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K132" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L132" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" spans="1:14">
+      <c r="A133" s="0">
+        <v>49415918</v>
+      </c>
+      <c r="B133" s="0" t="inlineStr">
+        <is>
+          <t>心语无言</t>
+        </is>
+      </c>
+      <c r="C133" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D133" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E133" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F133" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G133" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:24</t>
+        </is>
+      </c>
+      <c r="H133" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I133" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J133" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K133" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L133" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" spans="1:14">
+      <c r="A134" s="0">
+        <v>49415913</v>
+      </c>
+      <c r="B134" s="0" t="inlineStr">
+        <is>
+          <t>安好</t>
+        </is>
+      </c>
+      <c r="C134" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D134" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E134" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F134" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G134" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:18</t>
+        </is>
+      </c>
+      <c r="H134" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I134" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J134" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K134" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L134" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" spans="1:14">
+      <c r="A135" s="0">
+        <v>49415890</v>
+      </c>
+      <c r="B135" s="0" t="inlineStr">
+        <is>
+          <t>雨夜聆风</t>
+        </is>
+      </c>
+      <c r="C135" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D135" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E135" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F135" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G135" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:56</t>
+        </is>
+      </c>
+      <c r="H135" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I135" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J135" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K135" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L135" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="N135" s="0" t="inlineStr">
+        <is>
+          <t>宜春</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" spans="1:14">
+      <c r="A136" s="0">
+        <v>49415874</v>
+      </c>
+      <c r="B136" s="0" t="inlineStr">
+        <is>
+          <t>飘</t>
+        </is>
+      </c>
+      <c r="C136" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D136" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E136" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F136" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G136" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:40</t>
+        </is>
+      </c>
+      <c r="H136" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I136" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J136" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K136" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L136" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" spans="1:14">
+      <c r="A137" s="0">
+        <v>49415871</v>
+      </c>
+      <c r="B137" s="0" t="inlineStr">
+        <is>
+          <t>庆</t>
+        </is>
+      </c>
+      <c r="C137" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D137" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E137" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F137" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G137" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:36</t>
+        </is>
+      </c>
+      <c r="H137" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I137" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J137" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K137" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L137" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" spans="1:14">
+      <c r="A138" s="0">
         <v>49415867</v>
       </c>
-      <c r="B122" s="0" t="inlineStr">
+      <c r="B138" s="0" t="inlineStr">
         <is>
           <t>HYQ</t>
         </is>
       </c>
-      <c r="C122" s="0" t="inlineStr">
-        <is>
-          <t>6天0基础钢琴入门课</t>
-        </is>
-      </c>
-      <c r="D122" s="0" t="inlineStr">
-        <is>
-          <t>训练营</t>
-        </is>
-      </c>
-      <c r="E122" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="F122" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="G122" s="0" t="inlineStr">
+      <c r="C138" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D138" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E138" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F138" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G138" s="0" t="inlineStr">
         <is>
           <t>2026-08-19 22:47:33</t>
         </is>
       </c>
-      <c r="H122" s="0" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I122" s="0" t="inlineStr">
-        <is>
-          <t>黄老师-抖音01</t>
-        </is>
-      </c>
-      <c r="J122" s="0" t="inlineStr">
+      <c r="H138" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I138" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J138" s="0" t="inlineStr">
         <is>
           <t>安迪钢琴-多个点击报名-0元</t>
         </is>
       </c>
-      <c r="K122" s="0" t="inlineStr">
+      <c r="K138" s="0" t="inlineStr">
         <is>
           <t>微信支付</t>
         </is>
       </c>
-      <c r="L122" s="0" t="inlineStr">
+      <c r="L138" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>

</xml_diff>